<commit_message>
Updated tracker v4 and Invoice decion on 24 July
</commit_message>
<xml_diff>
--- a/files/Spinney_Budget_Tracker_v4.xlsx
+++ b/files/Spinney_Budget_Tracker_v4.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="177">
   <si>
     <t xml:space="preserve">Spinney External Works — Budget Summary</t>
   </si>
@@ -87,7 +87,7 @@
     <t xml:space="preserve">Chimney repair</t>
   </si>
   <si>
-    <t xml:space="preserve">Quoted separately (2 Jun). Labour £2,880 (10% discount, 20 Jul) no VAT + £80 rubbish; scaffolding £1,500 share of combined invoice; materials in pooled budget.</t>
+    <t xml:space="preserve">Quoted separately (2 Jun). Labour £3,200 no VAT (invoiced 24 Jul, full price — no cash discount) + £80 rubbish (outstanding) + scaffolding £1,500 share of combined invoice. Materials in pooled budget.</t>
   </si>
   <si>
     <t xml:space="preserve">Coping stones repair</t>
@@ -180,21 +180,24 @@
     <t xml:space="preserve">Log in Register: £562.50 chimney + £637.50 coping</t>
   </si>
   <si>
+    <t xml:space="preserve">INVOICED &amp; PAID 24 Jul (non-cash)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full price (invoiced, not cash): £3,200 labour + £80 rubbish = £3,280</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INVOICED &amp; PAID 24 Jul: £3,088.30 (labour less £111.70 prepaid). Rubbish £80 NOT yet invoiced — outstanding, follow up with Luke. Needs a couple more days on his return from holiday (timeline TBC, held for now).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Phase completion — SINGLE cash payment</t>
   </si>
   <si>
-    <t xml:space="preserve">Labour £2,880 (10% disc.) + rubbish £80 = £2,960; less £111.71 prepaid (work platform)</t>
+    <t xml:space="preserve">Labour £3,420 (10% disc.) + rubbish £80 = £3,500</t>
   </si>
   <si>
     <t xml:space="preserve">Lara/Ryan agreed — TBC Luke 21 Jul</t>
   </si>
   <si>
-    <t xml:space="preserve">CASH DUE ON COMPLETION: £2,848.29. One-week phase — no interim invoice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Labour £3,420 (10% disc.) + rubbish £80 = £3,500</t>
-  </si>
-  <si>
     <t xml:space="preserve">CASH DUE ON COMPLETION: £3,500.00</t>
   </si>
   <si>
@@ -294,7 +297,7 @@
     <t xml:space="preserve">LG invoice</t>
   </si>
   <si>
-    <t xml:space="preserve">Original quote £3,200; 10% labour discount agreed 20 Jul (Ryan/Luke): −£320</t>
+    <t xml:space="preserve">INVOICED 24 Jul (INV-0286), full price £3,200 less £111.70 prepaid = £3,088.30. Non-cash, so 10% discount does not apply. Rubbish removal £80 outstanding.</t>
   </si>
   <si>
     <t xml:space="preserve">Tubular scaffolding — all four sides of chimney and crown</t>
@@ -474,10 +477,28 @@
     <t xml:space="preserve">£2,000 paid following erection 17–18 Jul; amend date cell if payment day differed</t>
   </si>
   <si>
-    <t xml:space="preserve">Scaffold erection payment — coping share (pro-rata of £2,000 cash)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Balance £1,200 due on strike</t>
+    <t xml:space="preserve">INV-0286</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chimney labour, invoiced (£3,200 less £111.70 work-platform prepayment). Rubbish removal £80 NOT included — outstanding.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bank transfer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invoiced (non-cash) — full price, no 10% discount. £80 rubbish removal still outstanding.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dry Lining Supplies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">914751798</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weber Pral M Silver Pearl x10, Plastic 15mm Stop Bead 3m x3 (shared render finish)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Second pooled-materials trip</t>
   </si>
   <si>
     <t xml:space="preserve">Materials Receipts — pooled budget drawdown</t>
@@ -514,6 +535,12 @@
   </si>
   <si>
     <t xml:space="preserve">Render (chimney + coping, shared)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weber Pral M Silver Pearl x10 (£126.20), Plastic 15mm Stop Bead 3m x3 (£9.60), inc VAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Render finish (chimney + coping, shared)</t>
   </si>
   <si>
     <t xml:space="preserve">Contingency Drawdown — £5,000 pot (agreed Lara/Luke, 1 Jul 2026)</t>
@@ -747,7 +774,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -864,15 +891,7 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1299,19 +1318,19 @@
         <v>14</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>4460</v>
+        <v>4780</v>
       </c>
       <c r="D8" s="10" t="n">
         <f aca="false">SUMIF('Invoice Register'!$B:$B,$A8,'Invoice Register'!$F:$F)</f>
-        <v>1049.21</v>
+        <v>4137.51</v>
       </c>
       <c r="E8" s="10" t="n">
         <f aca="false">SUMIFS('Invoice Register'!$F:$F,'Invoice Register'!$B:$B,$A8,'Invoice Register'!$G:$G,"&lt;&gt;")</f>
-        <v>1049.21</v>
+        <v>4137.51</v>
       </c>
       <c r="F8" s="10" t="n">
         <f aca="false">C8-D8</f>
-        <v>3410.79</v>
+        <v>642.49</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>20</v>
@@ -1329,15 +1348,15 @@
       </c>
       <c r="D9" s="10" t="n">
         <f aca="false">SUMIF('Invoice Register'!$B:$B,$A9,'Invoice Register'!$F:$F)</f>
-        <v>1062.5</v>
+        <v>0</v>
       </c>
       <c r="E9" s="10" t="n">
         <f aca="false">SUMIFS('Invoice Register'!$F:$F,'Invoice Register'!$B:$B,$A9,'Invoice Register'!$G:$G,"&lt;&gt;")</f>
-        <v>1062.5</v>
+        <v>0</v>
       </c>
       <c r="F9" s="10" t="n">
         <f aca="false">C9-D9</f>
-        <v>4137.5</v>
+        <v>5200</v>
       </c>
       <c r="G9" s="12" t="s">
         <v>22</v>
@@ -1355,15 +1374,15 @@
       </c>
       <c r="D10" s="10" t="n">
         <f aca="false">SUMIF('Invoice Register'!$B:$B,$A10,'Invoice Register'!$F:$F)</f>
-        <v>311.98</v>
+        <v>474.94</v>
       </c>
       <c r="E10" s="10" t="n">
         <f aca="false">SUMIFS('Invoice Register'!$F:$F,'Invoice Register'!$B:$B,$A10,'Invoice Register'!$G:$G,"&lt;&gt;")</f>
-        <v>311.98</v>
+        <v>474.94</v>
       </c>
       <c r="F10" s="10" t="n">
         <f aca="false">C10-D10</f>
-        <v>818.02</v>
+        <v>655.06</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>25</v>
@@ -1399,19 +1418,19 @@
       <c r="B12" s="14"/>
       <c r="C12" s="15" t="n">
         <f aca="false">C8+C9+C10</f>
-        <v>10790</v>
+        <v>11110</v>
       </c>
       <c r="D12" s="15" t="n">
         <f aca="false">D8+D9+D10</f>
-        <v>2423.69</v>
+        <v>4612.45</v>
       </c>
       <c r="E12" s="15" t="n">
         <f aca="false">E8+E9+E10</f>
-        <v>2423.69</v>
+        <v>4612.45</v>
       </c>
       <c r="F12" s="15" t="n">
         <f aca="false">F8+F9+F10</f>
-        <v>8366.31</v>
+        <v>6497.55</v>
       </c>
       <c r="G12" s="14"/>
     </row>
@@ -1422,19 +1441,19 @@
       <c r="B13" s="17"/>
       <c r="C13" s="18" t="n">
         <f aca="false">C11+C12</f>
-        <v>66818.99</v>
+        <v>67138.99</v>
       </c>
       <c r="D13" s="18" t="n">
         <f aca="false">D11+D12</f>
-        <v>34652.68</v>
+        <v>36841.44</v>
       </c>
       <c r="E13" s="18" t="n">
         <f aca="false">E11+E12</f>
-        <v>34652.68</v>
+        <v>36841.44</v>
       </c>
       <c r="F13" s="18" t="n">
         <f aca="false">F11+F12</f>
-        <v>32166.31</v>
+        <v>30297.55</v>
       </c>
       <c r="G13" s="17"/>
     </row>
@@ -1607,13 +1626,13 @@
         <v>52</v>
       </c>
       <c r="F8" s="21" t="n">
-        <v>2960</v>
-      </c>
-      <c r="G8" s="24" t="s">
+        <v>3280</v>
+      </c>
+      <c r="G8" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="H8" s="8" t="s">
         <v>53</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1624,7 +1643,7 @@
         <v>21</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>14</v>
@@ -1636,10 +1655,10 @@
         <v>3500</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1650,22 +1669,22 @@
         <v>13</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>14</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F10" s="21" t="n">
         <v>18800</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1676,22 +1695,22 @@
         <v>23</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F11" s="21" t="n">
         <v>1130</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1702,22 +1721,22 @@
         <v>16</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F12" s="21" t="n">
         <v>5000</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1728,23 +1747,23 @@
         <v>23</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E13" s="25" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F13" s="26" t="n">
         <f aca="false">SUM(F5:F12)</f>
-        <v>66818.99</v>
+        <v>67138.99</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1755,28 +1774,28 @@
         <v>16</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F14" s="27" t="n">
         <f aca="false">Summary!$C$13</f>
-        <v>66818.99</v>
+        <v>67138.99</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E15" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F15" s="28" t="n">
         <f aca="false">F13-F14</f>
@@ -1784,34 +1803,22 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="29"/>
-      <c r="B16" s="29"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29"/>
-      <c r="E16" s="30" t="s">
-        <v>74</v>
-      </c>
-      <c r="F16" s="31" t="n">
+      <c r="E16" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F16" s="29" t="n">
         <f aca="false">Summary!$C$13</f>
-        <v>66818.99</v>
-      </c>
-      <c r="G16" s="29"/>
-      <c r="H16" s="29"/>
+        <v>67138.99</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="29"/>
-      <c r="B17" s="29"/>
-      <c r="C17" s="29"/>
-      <c r="D17" s="29"/>
-      <c r="E17" s="30" t="s">
-        <v>76</v>
-      </c>
-      <c r="F17" s="31" t="n">
+      <c r="E17" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="F17" s="29" t="n">
         <f aca="false">F15-F16</f>
-        <v>-66818.99</v>
-      </c>
-      <c r="G17" s="29"/>
-      <c r="H17" s="29"/>
+        <v>-67138.99</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1845,12 +1852,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1861,22 +1868,22 @@
         <v>4</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>9</v>
@@ -1887,24 +1894,24 @@
         <v>19</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
+        <v>87</v>
+      </c>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
       <c r="F5" s="21" t="n">
-        <v>2880</v>
-      </c>
-      <c r="G5" s="32" t="s">
-        <v>87</v>
+        <v>3200</v>
+      </c>
+      <c r="G5" s="30" t="s">
+        <v>88</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1915,21 +1922,21 @@
         <v>44</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32"/>
+        <v>91</v>
+      </c>
+      <c r="D6" s="30"/>
+      <c r="E6" s="30"/>
       <c r="F6" s="21" t="n">
         <v>1500</v>
       </c>
-      <c r="G6" s="32" t="s">
-        <v>91</v>
+      <c r="G6" s="30" t="s">
+        <v>92</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1940,18 +1947,18 @@
         <v>24</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
+        <v>95</v>
+      </c>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
       <c r="F7" s="21" t="n">
         <v>480</v>
       </c>
-      <c r="G7" s="32" t="s">
-        <v>91</v>
+      <c r="G7" s="30" t="s">
+        <v>92</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I7" s="11"/>
     </row>
@@ -1960,21 +1967,21 @@
         <v>19</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32"/>
+        <v>97</v>
+      </c>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
       <c r="F8" s="21" t="n">
         <v>80</v>
       </c>
-      <c r="G8" s="32" t="s">
-        <v>91</v>
+      <c r="G8" s="30" t="s">
+        <v>92</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I8" s="11"/>
     </row>
@@ -1983,24 +1990,24 @@
         <v>21</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32"/>
+        <v>98</v>
+      </c>
+      <c r="D9" s="30"/>
+      <c r="E9" s="30"/>
       <c r="F9" s="21" t="n">
         <v>3420</v>
       </c>
-      <c r="G9" s="32" t="s">
-        <v>87</v>
+      <c r="G9" s="30" t="s">
+        <v>88</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2011,21 +2018,21 @@
         <v>44</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32"/>
+        <v>100</v>
+      </c>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
       <c r="F10" s="21" t="n">
         <v>1700</v>
       </c>
-      <c r="G10" s="32" t="s">
-        <v>91</v>
+      <c r="G10" s="30" t="s">
+        <v>92</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2036,18 +2043,18 @@
         <v>24</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="D11" s="32"/>
-      <c r="E11" s="32"/>
+        <v>101</v>
+      </c>
+      <c r="D11" s="30"/>
+      <c r="E11" s="30"/>
       <c r="F11" s="21" t="n">
         <v>650</v>
       </c>
-      <c r="G11" s="32" t="s">
-        <v>91</v>
+      <c r="G11" s="30" t="s">
+        <v>92</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I11" s="11"/>
     </row>
@@ -2056,21 +2063,21 @@
         <v>21</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="D12" s="32"/>
-      <c r="E12" s="32"/>
+        <v>97</v>
+      </c>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30"/>
       <c r="F12" s="21" t="n">
         <v>80</v>
       </c>
-      <c r="G12" s="32" t="s">
-        <v>91</v>
+      <c r="G12" s="30" t="s">
+        <v>92</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I12" s="11"/>
     </row>
@@ -2079,24 +2086,24 @@
         <v>13</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="D13" s="32"/>
-      <c r="E13" s="32"/>
+        <v>102</v>
+      </c>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30"/>
       <c r="F13" s="21" t="n">
         <v>17600</v>
       </c>
-      <c r="G13" s="32" t="s">
-        <v>87</v>
+      <c r="G13" s="30" t="s">
+        <v>88</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I13" s="12" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2104,21 +2111,21 @@
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="D14" s="32"/>
-      <c r="E14" s="32"/>
+        <v>104</v>
+      </c>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
       <c r="F14" s="21" t="n">
         <v>1200</v>
       </c>
-      <c r="G14" s="32" t="s">
-        <v>91</v>
+      <c r="G14" s="30" t="s">
+        <v>92</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I14" s="11"/>
     </row>
@@ -2127,12 +2134,12 @@
         <v>10</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="D15" s="32" t="n">
+        <v>106</v>
+      </c>
+      <c r="D15" s="30" t="n">
         <v>230</v>
       </c>
       <c r="E15" s="21" t="n">
@@ -2141,11 +2148,11 @@
       <c r="F15" s="21" t="n">
         <v>15292.7</v>
       </c>
-      <c r="G15" s="32" t="s">
-        <v>106</v>
+      <c r="G15" s="30" t="s">
+        <v>107</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I15" s="11"/>
     </row>
@@ -2154,12 +2161,12 @@
         <v>10</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="D16" s="32" t="n">
+        <v>109</v>
+      </c>
+      <c r="D16" s="30" t="n">
         <v>18</v>
       </c>
       <c r="E16" s="21" t="n">
@@ -2168,11 +2175,11 @@
       <c r="F16" s="21" t="n">
         <v>1045.62</v>
       </c>
-      <c r="G16" s="32" t="s">
-        <v>106</v>
+      <c r="G16" s="30" t="s">
+        <v>107</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I16" s="11"/>
     </row>
@@ -2181,12 +2188,12 @@
         <v>10</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="D17" s="32" t="n">
+        <v>110</v>
+      </c>
+      <c r="D17" s="30" t="n">
         <v>15</v>
       </c>
       <c r="E17" s="21" t="n">
@@ -2195,14 +2202,14 @@
       <c r="F17" s="21" t="n">
         <v>1083.75</v>
       </c>
-      <c r="G17" s="32" t="s">
-        <v>106</v>
+      <c r="G17" s="30" t="s">
+        <v>107</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2210,12 +2217,12 @@
         <v>10</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="D18" s="32" t="n">
+        <v>112</v>
+      </c>
+      <c r="D18" s="30" t="n">
         <v>15</v>
       </c>
       <c r="E18" s="21" t="n">
@@ -2224,11 +2231,11 @@
       <c r="F18" s="21" t="n">
         <v>898.35</v>
       </c>
-      <c r="G18" s="32" t="s">
-        <v>106</v>
+      <c r="G18" s="30" t="s">
+        <v>107</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I18" s="11"/>
     </row>
@@ -2237,12 +2244,12 @@
         <v>10</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="D19" s="32" t="n">
+        <v>113</v>
+      </c>
+      <c r="D19" s="30" t="n">
         <v>24</v>
       </c>
       <c r="E19" s="21" t="n">
@@ -2251,11 +2258,11 @@
       <c r="F19" s="21" t="n">
         <v>770</v>
       </c>
-      <c r="G19" s="32" t="s">
-        <v>106</v>
+      <c r="G19" s="30" t="s">
+        <v>107</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I19" s="11"/>
     </row>
@@ -2264,12 +2271,12 @@
         <v>10</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="D20" s="32" t="n">
+        <v>114</v>
+      </c>
+      <c r="D20" s="30" t="n">
         <v>6</v>
       </c>
       <c r="E20" s="21" t="n">
@@ -2278,11 +2285,11 @@
       <c r="F20" s="21" t="n">
         <v>61.5</v>
       </c>
-      <c r="G20" s="32" t="s">
-        <v>106</v>
+      <c r="G20" s="30" t="s">
+        <v>107</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I20" s="11"/>
     </row>
@@ -2291,12 +2298,12 @@
         <v>10</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="D21" s="32" t="n">
+        <v>115</v>
+      </c>
+      <c r="D21" s="30" t="n">
         <v>266</v>
       </c>
       <c r="E21" s="21" t="n">
@@ -2305,14 +2312,14 @@
       <c r="F21" s="21" t="n">
         <v>7554.4</v>
       </c>
-      <c r="G21" s="32" t="s">
-        <v>106</v>
+      <c r="G21" s="30" t="s">
+        <v>107</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2320,12 +2327,12 @@
         <v>10</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="D22" s="32" t="n">
+        <v>117</v>
+      </c>
+      <c r="D22" s="30" t="n">
         <v>16</v>
       </c>
       <c r="E22" s="21" t="n">
@@ -2334,11 +2341,11 @@
       <c r="F22" s="21" t="n">
         <v>125.92</v>
       </c>
-      <c r="G22" s="32" t="s">
-        <v>106</v>
+      <c r="G22" s="30" t="s">
+        <v>107</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I22" s="11"/>
     </row>
@@ -2347,12 +2354,12 @@
         <v>10</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="D23" s="32" t="n">
+        <v>118</v>
+      </c>
+      <c r="D23" s="30" t="n">
         <v>1</v>
       </c>
       <c r="E23" s="21" t="n">
@@ -2361,11 +2368,11 @@
       <c r="F23" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="G23" s="32" t="s">
-        <v>106</v>
+      <c r="G23" s="30" t="s">
+        <v>107</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I23" s="11"/>
     </row>
@@ -2374,12 +2381,12 @@
         <v>10</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="D24" s="32" t="n">
+        <v>119</v>
+      </c>
+      <c r="D24" s="30" t="n">
         <v>1</v>
       </c>
       <c r="E24" s="21" t="n">
@@ -2388,11 +2395,11 @@
       <c r="F24" s="21" t="n">
         <v>10.25</v>
       </c>
-      <c r="G24" s="32" t="s">
-        <v>106</v>
+      <c r="G24" s="30" t="s">
+        <v>107</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I24" s="11"/>
     </row>
@@ -2401,24 +2408,24 @@
         <v>10</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="D25" s="32"/>
-      <c r="E25" s="32"/>
+        <v>120</v>
+      </c>
+      <c r="D25" s="30"/>
+      <c r="E25" s="30"/>
       <c r="F25" s="21" t="n">
         <v>5371.5</v>
       </c>
-      <c r="G25" s="32" t="s">
-        <v>83</v>
+      <c r="G25" s="30" t="s">
+        <v>84</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2426,33 +2433,33 @@
         <v>16</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="D26" s="32"/>
-      <c r="E26" s="32"/>
+        <v>123</v>
+      </c>
+      <c r="D26" s="30"/>
+      <c r="E26" s="30"/>
       <c r="F26" s="21" t="n">
         <v>5000</v>
       </c>
-      <c r="G26" s="32" t="s">
+      <c r="G26" s="30" t="s">
         <v>17</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C27" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="F27" s="34" t="n">
+      <c r="C27" s="31" t="s">
+        <v>126</v>
+      </c>
+      <c r="F27" s="32" t="n">
         <f aca="false">SUM(F5:F26)</f>
-        <v>66818.99</v>
+        <v>67138.99</v>
       </c>
     </row>
   </sheetData>
@@ -2485,17 +2492,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>3</v>
@@ -2504,26 +2511,26 @@
         <v>4</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="35" t="n">
+      <c r="A5" s="33" t="n">
         <v>46212</v>
       </c>
       <c r="B5" s="8" t="s">
@@ -2533,315 +2540,333 @@
         <v>11</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F5" s="21" t="n">
         <v>32228.99</v>
       </c>
-      <c r="G5" s="35" t="n">
+      <c r="G5" s="33" t="n">
         <v>46212</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="35" t="n">
+      <c r="A6" s="33" t="n">
         <v>46223</v>
       </c>
       <c r="B6" s="8" t="s">
         <v>23</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F6" s="21" t="n">
         <v>311.98</v>
       </c>
-      <c r="G6" s="35" t="n">
+      <c r="G6" s="33" t="n">
         <v>46223</v>
       </c>
       <c r="H6" s="20" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="35" t="n">
+      <c r="A7" s="33" t="n">
         <v>46223</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>19</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F7" s="21" t="n">
         <v>111.71</v>
       </c>
-      <c r="G7" s="35" t="n">
+      <c r="G7" s="33" t="n">
         <v>46223</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="35" t="n">
+      <c r="A8" s="33" t="n">
         <v>46223</v>
       </c>
       <c r="B8" s="8" t="s">
         <v>19</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F8" s="21" t="n">
         <v>937.5</v>
       </c>
-      <c r="G8" s="35" t="n">
+      <c r="G8" s="33" t="n">
         <v>46223</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="35" t="n">
-        <v>46223</v>
+      <c r="A9" s="33" t="n">
+        <v>46227</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>145</v>
+        <v>14</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F9" s="21" t="n">
-        <v>1062.5</v>
-      </c>
-      <c r="G9" s="35" t="n">
-        <v>46223</v>
+        <v>3088.3</v>
+      </c>
+      <c r="G9" s="33" t="n">
+        <v>46227</v>
       </c>
       <c r="H9" s="20" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="36"/>
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="37"/>
-      <c r="F10" s="38"/>
-      <c r="G10" s="36"/>
-      <c r="H10" s="37"/>
-      <c r="I10" s="37"/>
+      <c r="A10" s="33" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="F10" s="21" t="n">
+        <v>162.96</v>
+      </c>
+      <c r="G10" s="33" t="n">
+        <v>46225</v>
+      </c>
+      <c r="H10" s="20" t="s">
+        <v>142</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="36"/>
-      <c r="B11" s="37"/>
-      <c r="C11" s="37"/>
-      <c r="D11" s="37"/>
-      <c r="E11" s="37"/>
-      <c r="F11" s="38"/>
-      <c r="G11" s="36"/>
-      <c r="H11" s="37"/>
-      <c r="I11" s="37"/>
+      <c r="A11" s="34"/>
+      <c r="B11" s="35"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="35"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="34"/>
+      <c r="H11" s="35"/>
+      <c r="I11" s="35"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="36"/>
-      <c r="B12" s="37"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="37"/>
-      <c r="F12" s="38"/>
-      <c r="G12" s="36"/>
-      <c r="H12" s="37"/>
-      <c r="I12" s="37"/>
+      <c r="A12" s="34"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="36"/>
+      <c r="G12" s="34"/>
+      <c r="H12" s="35"/>
+      <c r="I12" s="35"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="36"/>
-      <c r="B13" s="37"/>
-      <c r="C13" s="37"/>
-      <c r="D13" s="37"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="38"/>
-      <c r="G13" s="36"/>
-      <c r="H13" s="37"/>
-      <c r="I13" s="37"/>
+      <c r="A13" s="34"/>
+      <c r="B13" s="35"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="35"/>
+      <c r="I13" s="35"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="36"/>
-      <c r="B14" s="37"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="37"/>
-      <c r="F14" s="38"/>
-      <c r="G14" s="36"/>
-      <c r="H14" s="37"/>
-      <c r="I14" s="37"/>
+      <c r="A14" s="34"/>
+      <c r="B14" s="35"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="34"/>
+      <c r="H14" s="35"/>
+      <c r="I14" s="35"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="36"/>
-      <c r="B15" s="37"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="38"/>
-      <c r="G15" s="36"/>
-      <c r="H15" s="37"/>
-      <c r="I15" s="37"/>
+      <c r="A15" s="34"/>
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="35"/>
+      <c r="I15" s="35"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="36"/>
-      <c r="B16" s="37"/>
-      <c r="C16" s="37"/>
-      <c r="D16" s="37"/>
-      <c r="E16" s="37"/>
-      <c r="F16" s="38"/>
-      <c r="G16" s="36"/>
-      <c r="H16" s="37"/>
-      <c r="I16" s="37"/>
+      <c r="A16" s="34"/>
+      <c r="B16" s="35"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="35"/>
+      <c r="E16" s="35"/>
+      <c r="F16" s="36"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="35"/>
+      <c r="I16" s="35"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="36"/>
-      <c r="B17" s="37"/>
-      <c r="C17" s="37"/>
-      <c r="D17" s="37"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="38"/>
-      <c r="G17" s="36"/>
-      <c r="H17" s="37"/>
-      <c r="I17" s="37"/>
+      <c r="A17" s="34"/>
+      <c r="B17" s="35"/>
+      <c r="C17" s="35"/>
+      <c r="D17" s="35"/>
+      <c r="E17" s="35"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="35"/>
+      <c r="I17" s="35"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="36"/>
-      <c r="B18" s="37"/>
-      <c r="C18" s="37"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="37"/>
-      <c r="F18" s="38"/>
-      <c r="G18" s="36"/>
-      <c r="H18" s="37"/>
-      <c r="I18" s="37"/>
+      <c r="A18" s="34"/>
+      <c r="B18" s="35"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="35"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="35"/>
+      <c r="I18" s="35"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="36"/>
-      <c r="B19" s="37"/>
-      <c r="C19" s="37"/>
-      <c r="D19" s="37"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="38"/>
-      <c r="G19" s="36"/>
-      <c r="H19" s="37"/>
-      <c r="I19" s="37"/>
+      <c r="A19" s="34"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="35"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="35"/>
+      <c r="I19" s="35"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="36"/>
-      <c r="B20" s="37"/>
-      <c r="C20" s="37"/>
-      <c r="D20" s="37"/>
-      <c r="E20" s="37"/>
-      <c r="F20" s="38"/>
-      <c r="G20" s="36"/>
-      <c r="H20" s="37"/>
-      <c r="I20" s="37"/>
+      <c r="A20" s="34"/>
+      <c r="B20" s="35"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="35"/>
+      <c r="E20" s="35"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="35"/>
+      <c r="I20" s="35"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="36"/>
-      <c r="B21" s="37"/>
-      <c r="C21" s="37"/>
-      <c r="D21" s="37"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="38"/>
-      <c r="G21" s="36"/>
-      <c r="H21" s="37"/>
-      <c r="I21" s="37"/>
+      <c r="A21" s="34"/>
+      <c r="B21" s="35"/>
+      <c r="C21" s="35"/>
+      <c r="D21" s="35"/>
+      <c r="E21" s="35"/>
+      <c r="F21" s="36"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="35"/>
+      <c r="I21" s="35"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="36"/>
-      <c r="B22" s="37"/>
-      <c r="C22" s="37"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="37"/>
-      <c r="F22" s="38"/>
-      <c r="G22" s="36"/>
-      <c r="H22" s="37"/>
-      <c r="I22" s="37"/>
+      <c r="A22" s="34"/>
+      <c r="B22" s="35"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="35"/>
+      <c r="E22" s="35"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="34"/>
+      <c r="H22" s="35"/>
+      <c r="I22" s="35"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="36"/>
-      <c r="B23" s="37"/>
-      <c r="C23" s="37"/>
-      <c r="D23" s="37"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="38"/>
-      <c r="G23" s="36"/>
-      <c r="H23" s="37"/>
-      <c r="I23" s="37"/>
+      <c r="A23" s="34"/>
+      <c r="B23" s="35"/>
+      <c r="C23" s="35"/>
+      <c r="D23" s="35"/>
+      <c r="E23" s="35"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="34"/>
+      <c r="H23" s="35"/>
+      <c r="I23" s="35"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="36"/>
-      <c r="B24" s="37"/>
-      <c r="C24" s="37"/>
-      <c r="D24" s="37"/>
-      <c r="E24" s="37"/>
-      <c r="F24" s="38"/>
-      <c r="G24" s="36"/>
-      <c r="H24" s="37"/>
-      <c r="I24" s="37"/>
+      <c r="A24" s="34"/>
+      <c r="B24" s="35"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="35"/>
+      <c r="E24" s="35"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="34"/>
+      <c r="H24" s="35"/>
+      <c r="I24" s="35"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="36"/>
-      <c r="B25" s="37"/>
-      <c r="C25" s="37"/>
-      <c r="D25" s="37"/>
-      <c r="E25" s="37"/>
-      <c r="F25" s="38"/>
-      <c r="G25" s="36"/>
-      <c r="H25" s="37"/>
-      <c r="I25" s="37"/>
+      <c r="A25" s="34"/>
+      <c r="B25" s="35"/>
+      <c r="C25" s="35"/>
+      <c r="D25" s="35"/>
+      <c r="E25" s="35"/>
+      <c r="F25" s="36"/>
+      <c r="G25" s="34"/>
+      <c r="H25" s="35"/>
+      <c r="I25" s="35"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2872,61 +2897,61 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="B4" s="39" t="n">
+        <v>160</v>
+      </c>
+      <c r="B4" s="37" t="n">
         <v>1130</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="D4" s="40" t="n">
+        <v>161</v>
+      </c>
+      <c r="D4" s="38" t="n">
         <f aca="false">B4-SUM(E8:E40)</f>
-        <v>818.02</v>
+        <v>655.06</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="35" t="n">
+      <c r="A8" s="33" t="n">
         <v>46223</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="E8" s="21" t="n">
         <v>311.98</v>
@@ -2937,187 +2962,197 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="36"/>
-      <c r="B9" s="37"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="38"/>
-      <c r="F9" s="10" t="str">
+      <c r="A9" s="33" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>170</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>171</v>
+      </c>
+      <c r="E9" s="21" t="n">
+        <v>162.96</v>
+      </c>
+      <c r="F9" s="10" t="n">
         <f aca="false">IF(E9="","",$B$4-SUM($E$8:E9))</f>
-        <v/>
+        <v>655.06</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="36"/>
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="38"/>
+      <c r="A10" s="34"/>
+      <c r="B10" s="35"/>
+      <c r="C10" s="35"/>
+      <c r="D10" s="35"/>
+      <c r="E10" s="36"/>
       <c r="F10" s="10" t="str">
         <f aca="false">IF(E10="","",$B$4-SUM($E$8:E10))</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="36"/>
-      <c r="B11" s="37"/>
-      <c r="C11" s="37"/>
-      <c r="D11" s="37"/>
-      <c r="E11" s="38"/>
+      <c r="A11" s="34"/>
+      <c r="B11" s="35"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="36"/>
       <c r="F11" s="10" t="str">
         <f aca="false">IF(E11="","",$B$4-SUM($E$8:E11))</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="36"/>
-      <c r="B12" s="37"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="38"/>
+      <c r="A12" s="34"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="36"/>
       <c r="F12" s="10" t="str">
         <f aca="false">IF(E12="","",$B$4-SUM($E$8:E12))</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="36"/>
-      <c r="B13" s="37"/>
-      <c r="C13" s="37"/>
-      <c r="D13" s="37"/>
-      <c r="E13" s="38"/>
+      <c r="A13" s="34"/>
+      <c r="B13" s="35"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="36"/>
       <c r="F13" s="10" t="str">
         <f aca="false">IF(E13="","",$B$4-SUM($E$8:E13))</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="36"/>
-      <c r="B14" s="37"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="38"/>
+      <c r="A14" s="34"/>
+      <c r="B14" s="35"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="36"/>
       <c r="F14" s="10" t="str">
         <f aca="false">IF(E14="","",$B$4-SUM($E$8:E14))</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="36"/>
-      <c r="B15" s="37"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="38"/>
+      <c r="A15" s="34"/>
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="36"/>
       <c r="F15" s="10" t="str">
         <f aca="false">IF(E15="","",$B$4-SUM($E$8:E15))</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="36"/>
-      <c r="B16" s="37"/>
-      <c r="C16" s="37"/>
-      <c r="D16" s="37"/>
-      <c r="E16" s="38"/>
+      <c r="A16" s="34"/>
+      <c r="B16" s="35"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="35"/>
+      <c r="E16" s="36"/>
       <c r="F16" s="10" t="str">
         <f aca="false">IF(E16="","",$B$4-SUM($E$8:E16))</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="36"/>
-      <c r="B17" s="37"/>
-      <c r="C17" s="37"/>
-      <c r="D17" s="37"/>
-      <c r="E17" s="38"/>
+      <c r="A17" s="34"/>
+      <c r="B17" s="35"/>
+      <c r="C17" s="35"/>
+      <c r="D17" s="35"/>
+      <c r="E17" s="36"/>
       <c r="F17" s="10" t="str">
         <f aca="false">IF(E17="","",$B$4-SUM($E$8:E17))</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="36"/>
-      <c r="B18" s="37"/>
-      <c r="C18" s="37"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="38"/>
+      <c r="A18" s="34"/>
+      <c r="B18" s="35"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="36"/>
       <c r="F18" s="10" t="str">
         <f aca="false">IF(E18="","",$B$4-SUM($E$8:E18))</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="36"/>
-      <c r="B19" s="37"/>
-      <c r="C19" s="37"/>
-      <c r="D19" s="37"/>
-      <c r="E19" s="38"/>
+      <c r="A19" s="34"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="36"/>
       <c r="F19" s="10" t="str">
         <f aca="false">IF(E19="","",$B$4-SUM($E$8:E19))</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="36"/>
-      <c r="B20" s="37"/>
-      <c r="C20" s="37"/>
-      <c r="D20" s="37"/>
-      <c r="E20" s="38"/>
+      <c r="A20" s="34"/>
+      <c r="B20" s="35"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="35"/>
+      <c r="E20" s="36"/>
       <c r="F20" s="10" t="str">
         <f aca="false">IF(E20="","",$B$4-SUM($E$8:E20))</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="36"/>
-      <c r="B21" s="37"/>
-      <c r="C21" s="37"/>
-      <c r="D21" s="37"/>
-      <c r="E21" s="38"/>
+      <c r="A21" s="34"/>
+      <c r="B21" s="35"/>
+      <c r="C21" s="35"/>
+      <c r="D21" s="35"/>
+      <c r="E21" s="36"/>
       <c r="F21" s="10" t="str">
         <f aca="false">IF(E21="","",$B$4-SUM($E$8:E21))</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="36"/>
-      <c r="B22" s="37"/>
-      <c r="C22" s="37"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="38"/>
+      <c r="A22" s="34"/>
+      <c r="B22" s="35"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="35"/>
+      <c r="E22" s="36"/>
       <c r="F22" s="10" t="str">
         <f aca="false">IF(E22="","",$B$4-SUM($E$8:E22))</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="36"/>
-      <c r="B23" s="37"/>
-      <c r="C23" s="37"/>
-      <c r="D23" s="37"/>
-      <c r="E23" s="38"/>
+      <c r="A23" s="34"/>
+      <c r="B23" s="35"/>
+      <c r="C23" s="35"/>
+      <c r="D23" s="35"/>
+      <c r="E23" s="36"/>
       <c r="F23" s="10" t="str">
         <f aca="false">IF(E23="","",$B$4-SUM($E$8:E23))</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="36"/>
-      <c r="B24" s="37"/>
-      <c r="C24" s="37"/>
-      <c r="D24" s="37"/>
-      <c r="E24" s="38"/>
+      <c r="A24" s="34"/>
+      <c r="B24" s="35"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="35"/>
+      <c r="E24" s="36"/>
       <c r="F24" s="10" t="str">
         <f aca="false">IF(E24="","",$B$4-SUM($E$8:E24))</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="36"/>
-      <c r="B25" s="37"/>
-      <c r="C25" s="37"/>
-      <c r="D25" s="37"/>
-      <c r="E25" s="38"/>
+      <c r="A25" s="34"/>
+      <c r="B25" s="35"/>
+      <c r="C25" s="35"/>
+      <c r="D25" s="35"/>
+      <c r="E25" s="36"/>
       <c r="F25" s="10" t="str">
         <f aca="false">IF(E25="","",$B$4-SUM($E$8:E25))</f>
         <v/>
@@ -3150,221 +3185,221 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="B4" s="39" t="n">
+        <v>174</v>
+      </c>
+      <c r="B4" s="37" t="n">
         <v>5000</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="D4" s="40" t="n">
+        <v>161</v>
+      </c>
+      <c r="D4" s="38" t="n">
         <f aca="false">B4-SUM(D8:D40)</f>
         <v>5000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="D7" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>160</v>
-      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="36"/>
-      <c r="B8" s="37"/>
-      <c r="C8" s="37"/>
-      <c r="D8" s="38"/>
+      <c r="A8" s="34"/>
+      <c r="B8" s="35"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="36"/>
       <c r="E8" s="10" t="str">
         <f aca="false">IF(D8="","",$B$4-SUM($D$8:D8))</f>
         <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="36"/>
-      <c r="B9" s="37"/>
-      <c r="C9" s="37"/>
-      <c r="D9" s="38"/>
+      <c r="A9" s="34"/>
+      <c r="B9" s="35"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="36"/>
       <c r="E9" s="10" t="str">
         <f aca="false">IF(D9="","",$B$4-SUM($D$8:D9))</f>
         <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="36"/>
-      <c r="B10" s="37"/>
-      <c r="C10" s="37"/>
-      <c r="D10" s="38"/>
+      <c r="A10" s="34"/>
+      <c r="B10" s="35"/>
+      <c r="C10" s="35"/>
+      <c r="D10" s="36"/>
       <c r="E10" s="10" t="str">
         <f aca="false">IF(D10="","",$B$4-SUM($D$8:D10))</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="36"/>
-      <c r="B11" s="37"/>
-      <c r="C11" s="37"/>
-      <c r="D11" s="38"/>
+      <c r="A11" s="34"/>
+      <c r="B11" s="35"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="36"/>
       <c r="E11" s="10" t="str">
         <f aca="false">IF(D11="","",$B$4-SUM($D$8:D11))</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="36"/>
-      <c r="B12" s="37"/>
-      <c r="C12" s="37"/>
-      <c r="D12" s="38"/>
+      <c r="A12" s="34"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="36"/>
       <c r="E12" s="10" t="str">
         <f aca="false">IF(D12="","",$B$4-SUM($D$8:D12))</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="36"/>
-      <c r="B13" s="37"/>
-      <c r="C13" s="37"/>
-      <c r="D13" s="38"/>
+      <c r="A13" s="34"/>
+      <c r="B13" s="35"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="36"/>
       <c r="E13" s="10" t="str">
         <f aca="false">IF(D13="","",$B$4-SUM($D$8:D13))</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="36"/>
-      <c r="B14" s="37"/>
-      <c r="C14" s="37"/>
-      <c r="D14" s="38"/>
+      <c r="A14" s="34"/>
+      <c r="B14" s="35"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="36"/>
       <c r="E14" s="10" t="str">
         <f aca="false">IF(D14="","",$B$4-SUM($D$8:D14))</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="36"/>
-      <c r="B15" s="37"/>
-      <c r="C15" s="37"/>
-      <c r="D15" s="38"/>
+      <c r="A15" s="34"/>
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="36"/>
       <c r="E15" s="10" t="str">
         <f aca="false">IF(D15="","",$B$4-SUM($D$8:D15))</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="36"/>
-      <c r="B16" s="37"/>
-      <c r="C16" s="37"/>
-      <c r="D16" s="38"/>
+      <c r="A16" s="34"/>
+      <c r="B16" s="35"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="36"/>
       <c r="E16" s="10" t="str">
         <f aca="false">IF(D16="","",$B$4-SUM($D$8:D16))</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="36"/>
-      <c r="B17" s="37"/>
-      <c r="C17" s="37"/>
-      <c r="D17" s="38"/>
+      <c r="A17" s="34"/>
+      <c r="B17" s="35"/>
+      <c r="C17" s="35"/>
+      <c r="D17" s="36"/>
       <c r="E17" s="10" t="str">
         <f aca="false">IF(D17="","",$B$4-SUM($D$8:D17))</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="36"/>
-      <c r="B18" s="37"/>
-      <c r="C18" s="37"/>
-      <c r="D18" s="38"/>
+      <c r="A18" s="34"/>
+      <c r="B18" s="35"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="36"/>
       <c r="E18" s="10" t="str">
         <f aca="false">IF(D18="","",$B$4-SUM($D$8:D18))</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="36"/>
-      <c r="B19" s="37"/>
-      <c r="C19" s="37"/>
-      <c r="D19" s="38"/>
+      <c r="A19" s="34"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="36"/>
       <c r="E19" s="10" t="str">
         <f aca="false">IF(D19="","",$B$4-SUM($D$8:D19))</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="36"/>
-      <c r="B20" s="37"/>
-      <c r="C20" s="37"/>
-      <c r="D20" s="38"/>
+      <c r="A20" s="34"/>
+      <c r="B20" s="35"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="36"/>
       <c r="E20" s="10" t="str">
         <f aca="false">IF(D20="","",$B$4-SUM($D$8:D20))</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="36"/>
-      <c r="B21" s="37"/>
-      <c r="C21" s="37"/>
-      <c r="D21" s="38"/>
+      <c r="A21" s="34"/>
+      <c r="B21" s="35"/>
+      <c r="C21" s="35"/>
+      <c r="D21" s="36"/>
       <c r="E21" s="10" t="str">
         <f aca="false">IF(D21="","",$B$4-SUM($D$8:D21))</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="36"/>
-      <c r="B22" s="37"/>
-      <c r="C22" s="37"/>
-      <c r="D22" s="38"/>
+      <c r="A22" s="34"/>
+      <c r="B22" s="35"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="36"/>
       <c r="E22" s="10" t="str">
         <f aca="false">IF(D22="","",$B$4-SUM($D$8:D22))</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="36"/>
-      <c r="B23" s="37"/>
-      <c r="C23" s="37"/>
-      <c r="D23" s="38"/>
+      <c r="A23" s="34"/>
+      <c r="B23" s="35"/>
+      <c r="C23" s="35"/>
+      <c r="D23" s="36"/>
       <c r="E23" s="10" t="str">
         <f aca="false">IF(D23="","",$B$4-SUM($D$8:D23))</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="36"/>
-      <c r="B24" s="37"/>
-      <c r="C24" s="37"/>
-      <c r="D24" s="38"/>
+      <c r="A24" s="34"/>
+      <c r="B24" s="35"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="36"/>
       <c r="E24" s="10" t="str">
         <f aca="false">IF(D24="","",$B$4-SUM($D$8:D24))</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="36"/>
-      <c r="B25" s="37"/>
-      <c r="C25" s="37"/>
-      <c r="D25" s="38"/>
+      <c r="A25" s="34"/>
+      <c r="B25" s="35"/>
+      <c r="C25" s="35"/>
+      <c r="D25" s="36"/>
       <c r="E25" s="10" t="str">
         <f aca="false">IF(D25="","",$B$4-SUM($D$8:D25))</f>
         <v/>

</xml_diff>

<commit_message>
Updated tracker to include materials receipt and new coping scope
Materials receipt added, new coping scopr work (5b) added to tracker and in decisions log
</commit_message>
<xml_diff>
--- a/files/Spinney_Budget_Tracker_v4.xlsx
+++ b/files/Spinney_Budget_Tracker_v4.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="190">
   <si>
     <t xml:space="preserve">Spinney External Works — Budget Summary</t>
   </si>
@@ -93,7 +93,7 @@
     <t xml:space="preserve">Coping stones repair</t>
   </si>
   <si>
-    <t xml:space="preserve">Quoted separately (3 Jun). Labour £3,420 (10% discount, 20 Jul) no VAT + £80 rubbish; scaffolding £1,700 share. RISK: damage to coping stones on removal could substantially increase cost. Materials in pooled budget.</t>
+    <t xml:space="preserve">Quoted separately (3 Jun). Labour £3,420 (10% discount, 20 Jul) no VAT + £80 rubbish; scaffolding £1,700 share; +£250 additional scope (condensation-escape prep, approved 4 Aug — cash/invoice split TBC). RISK: coping-stone damage on removal could substantially increase cost. Materials in pooled budget.</t>
   </si>
   <si>
     <t xml:space="preserve">Materials (pooled)</t>
@@ -201,6 +201,21 @@
     <t xml:space="preserve">CASH DUE ON COMPLETION: £3,500.00</t>
   </si>
   <si>
+    <t xml:space="preserve">5b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Additional scope — condensation-escape prep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Combined labour + materials estimate, per Luke's spec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved 4 Aug — cost split TBC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rebed 3 bricks, fibreglass mesh at parapet corners, 4 weep holes above damp-course membrane. Cash/invoice treatment (and 10% discount applicability) to confirm when Luke next onsite.</t>
+  </si>
+  <si>
     <t xml:space="preserve">4–5 stages — triggers TBC with Luke/Lara</t>
   </si>
   <si>
@@ -405,6 +420,15 @@
     <t xml:space="preserve">Track on Contingency Drawdown sheet. Labour invoices from this pot at 10% discount (extended 20 Jul); materials (cement/bricks) full price. Curved-decking extra labour: discount status TBC with Luke (decking exclusion boundary).</t>
   </si>
   <si>
+    <t xml:space="preserve">Additional scope — condensation-escape prep: re-bed 3 bricks; reinforce parapet corners with fibreglass mesh; fit 4 weep holes to front face above internal damp-course membrane (slate DPC capped in plastic DPM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Own line — pending resolution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved 4 Aug (spec from Luke received 5 Aug). Labour/materials split £250 combined estimate. Cash-vs-invoice treatment (and applicable 10% discount) NOT yet resolved — to confirm when Luke next onsite.</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOTAL (all lines)</t>
   </si>
   <si>
@@ -501,6 +525,15 @@
     <t xml:space="preserve">Second pooled-materials trip</t>
   </si>
   <si>
+    <t xml:space="preserve">RECB000NNIVB6DIPDFCW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weberend Ocr x3, Weber Pral M Silver Pearl x4, Stop Bead x6, Drip Bead x2, Sikabond SBR x1 (coping render)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coping stones render materials. Receipt received 4 Aug (till David, 07:31).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Materials Receipts — pooled budget drawdown</t>
   </si>
   <si>
@@ -541,6 +574,12 @@
   </si>
   <si>
     <t xml:space="preserve">Render finish (chimney + coping, shared)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weberend Ocr x3 (£29.13), Weber Pral M Silver Pearl x4 (£50.48), Stop Bead x6 (£19.20), Drip Bead x2 (£7.42), Sikabond SBR (£17.54), inc VAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Render (coping stones)</t>
   </si>
   <si>
     <t xml:space="preserve">Contingency Drawdown — £5,000 pot (agreed Lara/Luke, 1 Jul 2026)</t>
@@ -899,7 +938,7 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1203,7 +1242,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="n">
-        <v>46216</v>
+        <v>46238</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>2</v>
@@ -1344,7 +1383,7 @@
         <v>14</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>5200</v>
+        <v>5450</v>
       </c>
       <c r="D9" s="10" t="n">
         <f aca="false">SUMIF('Invoice Register'!$B:$B,$A9,'Invoice Register'!$F:$F)</f>
@@ -1356,7 +1395,7 @@
       </c>
       <c r="F9" s="10" t="n">
         <f aca="false">C9-D9</f>
-        <v>5200</v>
+        <v>5450</v>
       </c>
       <c r="G9" s="12" t="s">
         <v>22</v>
@@ -1374,15 +1413,15 @@
       </c>
       <c r="D10" s="10" t="n">
         <f aca="false">SUMIF('Invoice Register'!$B:$B,$A10,'Invoice Register'!$F:$F)</f>
-        <v>474.94</v>
+        <v>623.47</v>
       </c>
       <c r="E10" s="10" t="n">
         <f aca="false">SUMIFS('Invoice Register'!$F:$F,'Invoice Register'!$B:$B,$A10,'Invoice Register'!$G:$G,"&lt;&gt;")</f>
-        <v>474.94</v>
+        <v>623.47</v>
       </c>
       <c r="F10" s="10" t="n">
         <f aca="false">C10-D10</f>
-        <v>655.06</v>
+        <v>506.53</v>
       </c>
       <c r="G10" s="11" t="s">
         <v>25</v>
@@ -1418,19 +1457,19 @@
       <c r="B12" s="14"/>
       <c r="C12" s="15" t="n">
         <f aca="false">C8+C9+C10</f>
-        <v>11110</v>
+        <v>11360</v>
       </c>
       <c r="D12" s="15" t="n">
         <f aca="false">D8+D9+D10</f>
-        <v>4612.45</v>
+        <v>4760.98</v>
       </c>
       <c r="E12" s="15" t="n">
         <f aca="false">E8+E9+E10</f>
-        <v>4612.45</v>
+        <v>4760.98</v>
       </c>
       <c r="F12" s="15" t="n">
         <f aca="false">F8+F9+F10</f>
-        <v>6497.55</v>
+        <v>6599.02</v>
       </c>
       <c r="G12" s="14"/>
     </row>
@@ -1441,19 +1480,19 @@
       <c r="B13" s="17"/>
       <c r="C13" s="18" t="n">
         <f aca="false">C11+C12</f>
-        <v>67138.99</v>
+        <v>67388.99</v>
       </c>
       <c r="D13" s="18" t="n">
         <f aca="false">D11+D12</f>
-        <v>36841.44</v>
+        <v>36989.97</v>
       </c>
       <c r="E13" s="18" t="n">
         <f aca="false">E11+E12</f>
-        <v>36841.44</v>
+        <v>36989.97</v>
       </c>
       <c r="F13" s="18" t="n">
         <f aca="false">F11+F12</f>
-        <v>30297.55</v>
+        <v>30399.02</v>
       </c>
       <c r="G13" s="17"/>
     </row>
@@ -1483,7 +1522,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
@@ -1662,49 +1701,49 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="n">
-        <v>6</v>
+      <c r="A10" s="20" t="s">
+        <v>58</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>14</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F10" s="21" t="n">
-        <v>18800</v>
-      </c>
-      <c r="G10" s="23" t="s">
-        <v>60</v>
+        <v>250</v>
+      </c>
+      <c r="G10" s="24" t="s">
+        <v>61</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>63</v>
+        <v>14</v>
       </c>
       <c r="E11" s="8" t="s">
         <v>64</v>
       </c>
       <c r="F11" s="21" t="n">
-        <v>1130</v>
+        <v>18800</v>
       </c>
       <c r="G11" s="23" t="s">
         <v>65</v>
@@ -1715,10 +1754,10 @@
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>67</v>
@@ -1730,94 +1769,120 @@
         <v>69</v>
       </c>
       <c r="F12" s="21" t="n">
-        <v>5000</v>
+        <v>1130</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="E13" s="25" t="s">
-        <v>71</v>
-      </c>
-      <c r="F13" s="26" t="n">
-        <f aca="false">SUM(F5:F12)</f>
-        <v>67138.99</v>
+        <v>73</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="F13" s="21" t="n">
+        <v>5000</v>
       </c>
       <c r="G13" s="23" t="s">
         <v>65</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="E14" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="F14" s="26" t="n">
+        <f aca="false">SUM(F5:F13)</f>
+        <v>67388.99</v>
+      </c>
+      <c r="G14" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B15" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="F14" s="27" t="n">
+      <c r="C15" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="F15" s="27" t="n">
         <f aca="false">Summary!$C$13</f>
-        <v>67138.99</v>
-      </c>
-      <c r="G14" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E15" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="F15" s="28" t="n">
-        <f aca="false">F13-F14</f>
-        <v>0</v>
+        <v>67388.99</v>
+      </c>
+      <c r="G15" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E16" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F16" s="29" t="n">
-        <f aca="false">Summary!$C$13</f>
-        <v>67138.99</v>
+        <v>82</v>
+      </c>
+      <c r="F16" s="28" t="n">
+        <f aca="false">F14-F15</f>
+        <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E17" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="F17" s="29" t="n">
+        <f aca="false">Summary!$C$13</f>
+        <v>67388.99</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E18" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="F18" s="29" t="n">
         <f aca="false">F15-F16</f>
-        <v>-67138.99</v>
+        <v>67388.99</v>
       </c>
     </row>
   </sheetData>
@@ -1836,7 +1901,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
@@ -1852,12 +1917,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1868,22 +1933,22 @@
         <v>4</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>9</v>
@@ -1894,10 +1959,10 @@
         <v>19</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="D5" s="30"/>
       <c r="E5" s="30"/>
@@ -1905,13 +1970,13 @@
         <v>3200</v>
       </c>
       <c r="G5" s="30" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1922,7 +1987,7 @@
         <v>44</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="D6" s="30"/>
       <c r="E6" s="30"/>
@@ -1930,13 +1995,13 @@
         <v>1500</v>
       </c>
       <c r="G6" s="30" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1947,7 +2012,7 @@
         <v>24</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="D7" s="30"/>
       <c r="E7" s="30"/>
@@ -1955,10 +2020,10 @@
         <v>480</v>
       </c>
       <c r="G7" s="30" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I7" s="11"/>
     </row>
@@ -1967,10 +2032,10 @@
         <v>19</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D8" s="30"/>
       <c r="E8" s="30"/>
@@ -1978,10 +2043,10 @@
         <v>80</v>
       </c>
       <c r="G8" s="30" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="I8" s="11"/>
     </row>
@@ -1990,10 +2055,10 @@
         <v>21</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="D9" s="30"/>
       <c r="E9" s="30"/>
@@ -2001,13 +2066,13 @@
         <v>3420</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2018,7 +2083,7 @@
         <v>44</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D10" s="30"/>
       <c r="E10" s="30"/>
@@ -2026,13 +2091,13 @@
         <v>1700</v>
       </c>
       <c r="G10" s="30" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2043,7 +2108,7 @@
         <v>24</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D11" s="30"/>
       <c r="E11" s="30"/>
@@ -2051,10 +2116,10 @@
         <v>650</v>
       </c>
       <c r="G11" s="30" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I11" s="11"/>
     </row>
@@ -2063,10 +2128,10 @@
         <v>21</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D12" s="30"/>
       <c r="E12" s="30"/>
@@ -2074,10 +2139,10 @@
         <v>80</v>
       </c>
       <c r="G12" s="30" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="I12" s="11"/>
     </row>
@@ -2086,10 +2151,10 @@
         <v>13</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D13" s="30"/>
       <c r="E13" s="30"/>
@@ -2097,13 +2162,13 @@
         <v>17600</v>
       </c>
       <c r="G13" s="30" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="I13" s="12" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2111,10 +2176,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D14" s="30"/>
       <c r="E14" s="30"/>
@@ -2122,10 +2187,10 @@
         <v>1200</v>
       </c>
       <c r="G14" s="30" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="I14" s="11"/>
     </row>
@@ -2134,10 +2199,10 @@
         <v>10</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D15" s="30" t="n">
         <v>230</v>
@@ -2149,10 +2214,10 @@
         <v>15292.7</v>
       </c>
       <c r="G15" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I15" s="11"/>
     </row>
@@ -2161,10 +2226,10 @@
         <v>10</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D16" s="30" t="n">
         <v>18</v>
@@ -2176,10 +2241,10 @@
         <v>1045.62</v>
       </c>
       <c r="G16" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I16" s="11"/>
     </row>
@@ -2188,10 +2253,10 @@
         <v>10</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="D17" s="30" t="n">
         <v>15</v>
@@ -2203,13 +2268,13 @@
         <v>1083.75</v>
       </c>
       <c r="G17" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2217,10 +2282,10 @@
         <v>10</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="D18" s="30" t="n">
         <v>15</v>
@@ -2232,10 +2297,10 @@
         <v>898.35</v>
       </c>
       <c r="G18" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I18" s="11"/>
     </row>
@@ -2244,10 +2309,10 @@
         <v>10</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D19" s="30" t="n">
         <v>24</v>
@@ -2259,10 +2324,10 @@
         <v>770</v>
       </c>
       <c r="G19" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I19" s="11"/>
     </row>
@@ -2271,10 +2336,10 @@
         <v>10</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="D20" s="30" t="n">
         <v>6</v>
@@ -2286,10 +2351,10 @@
         <v>61.5</v>
       </c>
       <c r="G20" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I20" s="11"/>
     </row>
@@ -2298,10 +2363,10 @@
         <v>10</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D21" s="30" t="n">
         <v>266</v>
@@ -2313,13 +2378,13 @@
         <v>7554.4</v>
       </c>
       <c r="G21" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2327,10 +2392,10 @@
         <v>10</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D22" s="30" t="n">
         <v>16</v>
@@ -2342,10 +2407,10 @@
         <v>125.92</v>
       </c>
       <c r="G22" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I22" s="11"/>
     </row>
@@ -2354,10 +2419,10 @@
         <v>10</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="D23" s="30" t="n">
         <v>1</v>
@@ -2369,10 +2434,10 @@
         <v>15</v>
       </c>
       <c r="G23" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I23" s="11"/>
     </row>
@@ -2381,10 +2446,10 @@
         <v>10</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D24" s="30" t="n">
         <v>1</v>
@@ -2396,10 +2461,10 @@
         <v>10.25</v>
       </c>
       <c r="G24" s="30" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I24" s="11"/>
     </row>
@@ -2408,10 +2473,10 @@
         <v>10</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="D25" s="30"/>
       <c r="E25" s="30"/>
@@ -2419,13 +2484,13 @@
         <v>5371.5</v>
       </c>
       <c r="G25" s="30" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2433,10 +2498,10 @@
         <v>16</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D26" s="30"/>
       <c r="E26" s="30"/>
@@ -2447,19 +2512,44 @@
         <v>17</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C27" s="31" t="s">
-        <v>126</v>
-      </c>
-      <c r="F27" s="32" t="n">
-        <f aca="false">SUM(F5:F26)</f>
-        <v>67138.99</v>
+      <c r="A27" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="D27" s="30"/>
+      <c r="E27" s="30"/>
+      <c r="F27" s="21" t="n">
+        <v>250</v>
+      </c>
+      <c r="G27" s="30" t="s">
+        <v>127</v>
+      </c>
+      <c r="H27" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="I27" s="8" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C28" s="31" t="s">
+        <v>134</v>
+      </c>
+      <c r="F28" s="32" t="n">
+        <f aca="false">SUM(F5:F27)</f>
+        <v>67388.99</v>
       </c>
     </row>
   </sheetData>
@@ -2492,17 +2582,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>3</v>
@@ -2511,19 +2601,19 @@
         <v>4</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>9</v>
@@ -2540,10 +2630,10 @@
         <v>11</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="F5" s="21" t="n">
         <v>32228.99</v>
@@ -2552,10 +2642,10 @@
         <v>46212</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2566,13 +2656,13 @@
         <v>23</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="F6" s="21" t="n">
         <v>311.98</v>
@@ -2581,10 +2671,10 @@
         <v>46223</v>
       </c>
       <c r="H6" s="20" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2595,13 +2685,13 @@
         <v>19</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="F7" s="21" t="n">
         <v>111.71</v>
@@ -2610,10 +2700,10 @@
         <v>46223</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2624,13 +2714,13 @@
         <v>19</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="F8" s="21" t="n">
         <v>937.5</v>
@@ -2639,10 +2729,10 @@
         <v>46223</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2656,10 +2746,10 @@
         <v>14</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="F9" s="21" t="n">
         <v>3088.3</v>
@@ -2668,10 +2758,10 @@
         <v>46227</v>
       </c>
       <c r="H9" s="20" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2682,13 +2772,13 @@
         <v>23</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="F10" s="21" t="n">
         <v>162.96</v>
@@ -2697,22 +2787,40 @@
         <v>46225</v>
       </c>
       <c r="H10" s="20" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="34"/>
-      <c r="B11" s="35"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="36"/>
-      <c r="G11" s="34"/>
-      <c r="H11" s="35"/>
-      <c r="I11" s="35"/>
+      <c r="A11" s="33" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="F11" s="21" t="n">
+        <v>148.53</v>
+      </c>
+      <c r="G11" s="33" t="n">
+        <v>46238</v>
+      </c>
+      <c r="H11" s="20" t="s">
+        <v>150</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>168</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="34"/>
@@ -2897,47 +3005,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>158</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="B4" s="37" t="n">
         <v>1130</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="D4" s="38" t="n">
         <f aca="false">B4-SUM(E8:E40)</f>
-        <v>655.06</v>
+        <v>506.53</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2945,13 +3053,13 @@
         <v>46223</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>168</v>
+        <v>179</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
       <c r="E8" s="21" t="n">
         <v>311.98</v>
@@ -2966,13 +3074,13 @@
         <v>46225</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="E9" s="21" t="n">
         <v>162.96</v>
@@ -2983,14 +3091,24 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="34"/>
-      <c r="B10" s="35"/>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="10" t="str">
+      <c r="A10" s="33" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>184</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>148.53</v>
+      </c>
+      <c r="F10" s="10" t="n">
         <f aca="false">IF(E10="","",$B$4-SUM($E$8:E10))</f>
-        <v/>
+        <v>506.53</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3185,23 +3303,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="B4" s="37" t="n">
         <v>5000</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="D4" s="38" t="n">
         <f aca="false">B4-SUM(D8:D40)</f>
@@ -3210,19 +3328,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Decision log updated - new chimney cowl, coping cash paid
</commit_message>
<xml_diff>
--- a/files/Spinney_Budget_Tracker_v4.xlsx
+++ b/files/Spinney_Budget_Tracker_v4.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="196">
   <si>
     <t xml:space="preserve">Spinney External Works — Budget Summary</t>
   </si>
@@ -93,7 +93,7 @@
     <t xml:space="preserve">Coping stones repair</t>
   </si>
   <si>
-    <t xml:space="preserve">Quoted separately (3 Jun). Labour £3,420 (10% discount, 20 Jul) no VAT + £80 rubbish; scaffolding £1,700 share; +£250 additional scope (condensation-escape prep, approved 4 Aug — cash/invoice split TBC). RISK: coping-stone damage on removal could substantially increase cost. Materials in pooled budget.</t>
+    <t xml:space="preserve">Quoted separately (3 Jun). Base labour blended, confirmed 7 Aug: 50% cash (10% disc.) + 50% invoiced = £3610.00. +£80 rubbish (full price, rides with invoice portion). +£1,700 scaffold share. +£250 condensation-prep addition — PRICE NOT FINALISED, terms will be 100% cash + materials, separate from this split. RISK: coping-stone damage on removal could substantially increase cost. Materials in pooled budget.</t>
   </si>
   <si>
     <t xml:space="preserve">Materials (pooled)</t>
@@ -189,31 +189,43 @@
     <t xml:space="preserve">INVOICED &amp; PAID 24 Jul: £3,088.30 (labour less £111.70 prepaid). Rubbish £80 NOT yet invoiced — outstanding, follow up with Luke. Needs a couple more days on his return from holiday (timeline TBC, held for now).</t>
   </si>
   <si>
-    <t xml:space="preserve">Phase completion — SINGLE cash payment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Labour £3,420 (10% disc.) + rubbish £80 = £3,500</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lara/Ryan agreed — TBC Luke 21 Jul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CASH DUE ON COMPLETION: £3,500.00</t>
+    <t xml:space="preserve">50% CASH — due today, 7 Aug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50% of base labour (£1710.00), 10% cash discount applied. Based on original £3,800 quote only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Due today</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONFIRMED 7 Aug. Excludes condensation-prep addition — its price is not yet finalised (see separate row).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50% INVOICED — due next week</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50% of base labour (£1900.00) full price, + £80 rubbish removal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved 7 Aug — awaiting invoice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rubbish removal assumed to ride with this invoice (unconfirmed — chimney's £80 is still outstanding as a comparator).</t>
   </si>
   <si>
     <t xml:space="preserve">5b</t>
   </si>
   <si>
-    <t xml:space="preserve">Additional scope — condensation-escape prep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Combined labour + materials estimate, per Luke's spec</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Approved 4 Aug — cost split TBC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rebed 3 bricks, fibreglass mesh at parapet corners, 4 weep holes above damp-course membrane. Cash/invoice treatment (and 10% discount applicability) to confirm when Luke next onsite.</t>
+    <t xml:space="preserve">Additional scope — condensation-escape prep (price TBC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Combined labour + materials, Luke's estimate — price NOT yet finalised</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price TBC — not finalised (7 Aug)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terms confirmed 7 Aug: 100% cash (labour + materials) once priced. Separate from the base coping 50/50 split. £250 is provisional.</t>
   </si>
   <si>
     <t xml:space="preserve">4–5 stages — triggers TBC with Luke/Lara</t>
@@ -339,7 +351,7 @@
     <t xml:space="preserve">Labour — remove/reset copings, slate cap, render, lead flashings to parapet rear</t>
   </si>
   <si>
-    <t xml:space="preserve">Original quote £3,800; 10% labour discount agreed 20 Jul (Ryan/Luke): −£380. RISK: stone damage on removal could substantially increase cost</t>
+    <t xml:space="preserve">CONFIRMED 7 Aug, based on original £3,800 quote: 50% cash (£1710.00 @ 10% discount) due same day, 50% invoiced (£1900.00 full price) due next week. RISK: coping-stone damage on removal could substantially increase cost.</t>
   </si>
   <si>
     <t xml:space="preserve">Tubular scaffolding with winch system</t>
@@ -426,7 +438,7 @@
     <t xml:space="preserve">Own line — pending resolution</t>
   </si>
   <si>
-    <t xml:space="preserve">Approved 4 Aug (spec from Luke received 5 Aug). Labour/materials split £250 combined estimate. Cash-vs-invoice treatment (and applicable 10% discount) NOT yet resolved — to confirm when Luke next onsite.</t>
+    <t xml:space="preserve">PRICE NOT YET FINALISED (7 Aug). Terms confirmed: 100% cash (labour + materials) once priced — separate from the base coping 50/50 split. £250 is Luke's original estimate only; treat as provisional until a firm figure is given.</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL (all lines)</t>
@@ -532,6 +544,12 @@
   </si>
   <si>
     <t xml:space="preserve">Coping stones render materials. Receipt received 4 Aug (till David, 07:31).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coping 50% cash labour payment (base labour only, 10% discount). Condensation-prep addition NOT included — price not yet finalised.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmed 7 Aug: 50% cash / 50% invoice split on original £3,800 quote. Remainder £1,980.00 (incl. rubbish) to be invoiced next week. £250 addition separate, price TBC.</t>
   </si>
   <si>
     <t xml:space="preserve">Materials Receipts — pooled budget drawdown</t>
@@ -813,7 +831,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="42">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -930,6 +948,18 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -938,7 +968,7 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1242,7 +1272,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="n">
-        <v>46238</v>
+        <v>46241</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>2</v>
@@ -1383,19 +1413,19 @@
         <v>14</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>5450</v>
+        <v>5640</v>
       </c>
       <c r="D9" s="10" t="n">
         <f aca="false">SUMIF('Invoice Register'!$B:$B,$A9,'Invoice Register'!$F:$F)</f>
-        <v>0</v>
+        <v>1710</v>
       </c>
       <c r="E9" s="10" t="n">
         <f aca="false">SUMIFS('Invoice Register'!$F:$F,'Invoice Register'!$B:$B,$A9,'Invoice Register'!$G:$G,"&lt;&gt;")</f>
-        <v>0</v>
+        <v>1710</v>
       </c>
       <c r="F9" s="10" t="n">
         <f aca="false">C9-D9</f>
-        <v>5450</v>
+        <v>3930</v>
       </c>
       <c r="G9" s="12" t="s">
         <v>22</v>
@@ -1457,19 +1487,19 @@
       <c r="B12" s="14"/>
       <c r="C12" s="15" t="n">
         <f aca="false">C8+C9+C10</f>
-        <v>11360</v>
+        <v>11550</v>
       </c>
       <c r="D12" s="15" t="n">
         <f aca="false">D8+D9+D10</f>
-        <v>4760.98</v>
+        <v>6470.98</v>
       </c>
       <c r="E12" s="15" t="n">
         <f aca="false">E8+E9+E10</f>
-        <v>4760.98</v>
+        <v>6470.98</v>
       </c>
       <c r="F12" s="15" t="n">
         <f aca="false">F8+F9+F10</f>
-        <v>6599.02</v>
+        <v>5079.02</v>
       </c>
       <c r="G12" s="14"/>
     </row>
@@ -1480,19 +1510,19 @@
       <c r="B13" s="17"/>
       <c r="C13" s="18" t="n">
         <f aca="false">C11+C12</f>
-        <v>67388.99</v>
+        <v>67578.99</v>
       </c>
       <c r="D13" s="18" t="n">
         <f aca="false">D11+D12</f>
-        <v>36989.97</v>
+        <v>38699.97</v>
       </c>
       <c r="E13" s="18" t="n">
         <f aca="false">E11+E12</f>
-        <v>36989.97</v>
+        <v>38699.97</v>
       </c>
       <c r="F13" s="18" t="n">
         <f aca="false">F11+F12</f>
-        <v>30399.02</v>
+        <v>28879.02</v>
       </c>
       <c r="G13" s="17"/>
     </row>
@@ -1522,7 +1552,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
@@ -1691,7 +1721,7 @@
         <v>55</v>
       </c>
       <c r="F9" s="21" t="n">
-        <v>3500</v>
+        <v>1710</v>
       </c>
       <c r="G9" s="24" t="s">
         <v>56</v>
@@ -1701,37 +1731,37 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
-        <v>58</v>
+      <c r="A10" s="20" t="n">
+        <v>6</v>
       </c>
       <c r="B10" s="8" t="s">
         <v>21</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>14</v>
       </c>
       <c r="E10" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="F10" s="21" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G10" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="F10" s="21" t="n">
-        <v>250</v>
-      </c>
-      <c r="G10" s="24" t="s">
+      <c r="H10" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="H10" s="8" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="20" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="n">
-        <v>6</v>
-      </c>
       <c r="B11" s="8" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>63</v>
@@ -1743,9 +1773,9 @@
         <v>64</v>
       </c>
       <c r="F11" s="21" t="n">
-        <v>18800</v>
-      </c>
-      <c r="G11" s="23" t="s">
+        <v>250</v>
+      </c>
+      <c r="G11" s="24" t="s">
         <v>65</v>
       </c>
       <c r="H11" s="8" t="s">
@@ -1754,51 +1784,51 @@
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>67</v>
       </c>
       <c r="D12" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="F12" s="21" t="n">
+        <v>18800</v>
+      </c>
+      <c r="G12" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="F12" s="21" t="n">
-        <v>1130</v>
-      </c>
-      <c r="G12" s="23" t="s">
+      <c r="H12" s="8" t="s">
         <v>70</v>
-      </c>
-      <c r="H12" s="8" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C13" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="E13" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="F13" s="21" t="n">
+        <v>1130</v>
+      </c>
+      <c r="G13" s="23" t="s">
         <v>74</v>
-      </c>
-      <c r="F13" s="21" t="n">
-        <v>5000</v>
-      </c>
-      <c r="G13" s="23" t="s">
-        <v>65</v>
       </c>
       <c r="H13" s="8" t="s">
         <v>75</v>
@@ -1806,83 +1836,115 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="E14" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="F14" s="26" t="n">
-        <f aca="false">SUM(F5:F13)</f>
-        <v>67388.99</v>
+        <v>77</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="F14" s="21" t="n">
+        <v>5000</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="E15" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E15" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="F15" s="27" t="n">
-        <f aca="false">Summary!$C$13</f>
-        <v>67388.99</v>
+      <c r="F15" s="26" t="n">
+        <f aca="false">SUM(F5:F14)</f>
+        <v>67578.99</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="H15" s="8" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E16" s="3" t="s">
+      <c r="A16" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="F16" s="28" t="n">
-        <f aca="false">F14-F15</f>
-        <v>0</v>
+      <c r="D16" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="F16" s="27" t="n">
+        <f aca="false">Summary!$C$13</f>
+        <v>67578.99</v>
+      </c>
+      <c r="G16" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E17" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="F17" s="29" t="n">
+        <v>86</v>
+      </c>
+      <c r="F17" s="28" t="n">
+        <f aca="false">F15-F16</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="29"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="F18" s="31" t="n">
         <f aca="false">Summary!$C$13</f>
-        <v>67388.99</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E18" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="F18" s="29" t="n">
+        <v>67578.99</v>
+      </c>
+      <c r="G18" s="29"/>
+      <c r="H18" s="29"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E19" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F19" s="32" t="n">
         <f aca="false">F15-F16</f>
-        <v>67388.99</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1917,12 +1979,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1933,22 +1995,22 @@
         <v>4</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>9</v>
@@ -1959,24 +2021,24 @@
         <v>19</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
+        <v>96</v>
+      </c>
+      <c r="D5" s="33"/>
+      <c r="E5" s="33"/>
       <c r="F5" s="21" t="n">
         <v>3200</v>
       </c>
-      <c r="G5" s="30" t="s">
-        <v>93</v>
+      <c r="G5" s="33" t="s">
+        <v>97</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1987,21 +2049,21 @@
         <v>44</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="D6" s="30"/>
-      <c r="E6" s="30"/>
+        <v>100</v>
+      </c>
+      <c r="D6" s="33"/>
+      <c r="E6" s="33"/>
       <c r="F6" s="21" t="n">
         <v>1500</v>
       </c>
-      <c r="G6" s="30" t="s">
-        <v>97</v>
+      <c r="G6" s="33" t="s">
+        <v>101</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2012,18 +2074,18 @@
         <v>24</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="D7" s="30"/>
-      <c r="E7" s="30"/>
+        <v>104</v>
+      </c>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
       <c r="F7" s="21" t="n">
         <v>480</v>
       </c>
-      <c r="G7" s="30" t="s">
-        <v>97</v>
+      <c r="G7" s="33" t="s">
+        <v>101</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="I7" s="11"/>
     </row>
@@ -2032,21 +2094,21 @@
         <v>19</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
+        <v>106</v>
+      </c>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
       <c r="F8" s="21" t="n">
         <v>80</v>
       </c>
-      <c r="G8" s="30" t="s">
-        <v>97</v>
+      <c r="G8" s="33" t="s">
+        <v>101</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="I8" s="11"/>
     </row>
@@ -2055,24 +2117,24 @@
         <v>21</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="D9" s="30"/>
-      <c r="E9" s="30"/>
+        <v>107</v>
+      </c>
+      <c r="D9" s="33"/>
+      <c r="E9" s="33"/>
       <c r="F9" s="21" t="n">
-        <v>3420</v>
-      </c>
-      <c r="G9" s="30" t="s">
-        <v>93</v>
+        <v>3610</v>
+      </c>
+      <c r="G9" s="33" t="s">
+        <v>97</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2083,21 +2145,21 @@
         <v>44</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="D10" s="30"/>
-      <c r="E10" s="30"/>
+        <v>109</v>
+      </c>
+      <c r="D10" s="33"/>
+      <c r="E10" s="33"/>
       <c r="F10" s="21" t="n">
         <v>1700</v>
       </c>
-      <c r="G10" s="30" t="s">
-        <v>97</v>
+      <c r="G10" s="33" t="s">
+        <v>101</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2108,18 +2170,18 @@
         <v>24</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="D11" s="30"/>
-      <c r="E11" s="30"/>
+        <v>110</v>
+      </c>
+      <c r="D11" s="33"/>
+      <c r="E11" s="33"/>
       <c r="F11" s="21" t="n">
         <v>650</v>
       </c>
-      <c r="G11" s="30" t="s">
-        <v>97</v>
+      <c r="G11" s="33" t="s">
+        <v>101</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="I11" s="11"/>
     </row>
@@ -2128,21 +2190,21 @@
         <v>21</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
+        <v>106</v>
+      </c>
+      <c r="D12" s="33"/>
+      <c r="E12" s="33"/>
       <c r="F12" s="21" t="n">
         <v>80</v>
       </c>
-      <c r="G12" s="30" t="s">
-        <v>97</v>
+      <c r="G12" s="33" t="s">
+        <v>101</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="I12" s="11"/>
     </row>
@@ -2151,24 +2213,24 @@
         <v>13</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="D13" s="30"/>
-      <c r="E13" s="30"/>
+        <v>111</v>
+      </c>
+      <c r="D13" s="33"/>
+      <c r="E13" s="33"/>
       <c r="F13" s="21" t="n">
         <v>17600</v>
       </c>
-      <c r="G13" s="30" t="s">
-        <v>93</v>
+      <c r="G13" s="33" t="s">
+        <v>97</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="I13" s="12" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2176,21 +2238,21 @@
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="D14" s="30"/>
-      <c r="E14" s="30"/>
+        <v>113</v>
+      </c>
+      <c r="D14" s="33"/>
+      <c r="E14" s="33"/>
       <c r="F14" s="21" t="n">
         <v>1200</v>
       </c>
-      <c r="G14" s="30" t="s">
-        <v>97</v>
+      <c r="G14" s="33" t="s">
+        <v>101</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="I14" s="11"/>
     </row>
@@ -2199,12 +2261,12 @@
         <v>10</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="D15" s="30" t="n">
+        <v>115</v>
+      </c>
+      <c r="D15" s="33" t="n">
         <v>230</v>
       </c>
       <c r="E15" s="21" t="n">
@@ -2213,11 +2275,11 @@
       <c r="F15" s="21" t="n">
         <v>15292.7</v>
       </c>
-      <c r="G15" s="30" t="s">
-        <v>112</v>
+      <c r="G15" s="33" t="s">
+        <v>116</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I15" s="11"/>
     </row>
@@ -2226,12 +2288,12 @@
         <v>10</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="D16" s="30" t="n">
+        <v>118</v>
+      </c>
+      <c r="D16" s="33" t="n">
         <v>18</v>
       </c>
       <c r="E16" s="21" t="n">
@@ -2240,11 +2302,11 @@
       <c r="F16" s="21" t="n">
         <v>1045.62</v>
       </c>
-      <c r="G16" s="30" t="s">
-        <v>112</v>
+      <c r="G16" s="33" t="s">
+        <v>116</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I16" s="11"/>
     </row>
@@ -2253,12 +2315,12 @@
         <v>10</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="D17" s="30" t="n">
+        <v>119</v>
+      </c>
+      <c r="D17" s="33" t="n">
         <v>15</v>
       </c>
       <c r="E17" s="21" t="n">
@@ -2267,14 +2329,14 @@
       <c r="F17" s="21" t="n">
         <v>1083.75</v>
       </c>
-      <c r="G17" s="30" t="s">
-        <v>112</v>
+      <c r="G17" s="33" t="s">
+        <v>116</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2282,12 +2344,12 @@
         <v>10</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="D18" s="30" t="n">
+        <v>121</v>
+      </c>
+      <c r="D18" s="33" t="n">
         <v>15</v>
       </c>
       <c r="E18" s="21" t="n">
@@ -2296,11 +2358,11 @@
       <c r="F18" s="21" t="n">
         <v>898.35</v>
       </c>
-      <c r="G18" s="30" t="s">
-        <v>112</v>
+      <c r="G18" s="33" t="s">
+        <v>116</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I18" s="11"/>
     </row>
@@ -2309,12 +2371,12 @@
         <v>10</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="D19" s="30" t="n">
+        <v>122</v>
+      </c>
+      <c r="D19" s="33" t="n">
         <v>24</v>
       </c>
       <c r="E19" s="21" t="n">
@@ -2323,11 +2385,11 @@
       <c r="F19" s="21" t="n">
         <v>770</v>
       </c>
-      <c r="G19" s="30" t="s">
-        <v>112</v>
+      <c r="G19" s="33" t="s">
+        <v>116</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I19" s="11"/>
     </row>
@@ -2336,12 +2398,12 @@
         <v>10</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="D20" s="30" t="n">
+        <v>123</v>
+      </c>
+      <c r="D20" s="33" t="n">
         <v>6</v>
       </c>
       <c r="E20" s="21" t="n">
@@ -2350,11 +2412,11 @@
       <c r="F20" s="21" t="n">
         <v>61.5</v>
       </c>
-      <c r="G20" s="30" t="s">
-        <v>112</v>
+      <c r="G20" s="33" t="s">
+        <v>116</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I20" s="11"/>
     </row>
@@ -2363,12 +2425,12 @@
         <v>10</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="D21" s="30" t="n">
+        <v>124</v>
+      </c>
+      <c r="D21" s="33" t="n">
         <v>266</v>
       </c>
       <c r="E21" s="21" t="n">
@@ -2377,14 +2439,14 @@
       <c r="F21" s="21" t="n">
         <v>7554.4</v>
       </c>
-      <c r="G21" s="30" t="s">
-        <v>112</v>
+      <c r="G21" s="33" t="s">
+        <v>116</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2392,12 +2454,12 @@
         <v>10</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="D22" s="30" t="n">
+        <v>126</v>
+      </c>
+      <c r="D22" s="33" t="n">
         <v>16</v>
       </c>
       <c r="E22" s="21" t="n">
@@ -2406,11 +2468,11 @@
       <c r="F22" s="21" t="n">
         <v>125.92</v>
       </c>
-      <c r="G22" s="30" t="s">
-        <v>112</v>
+      <c r="G22" s="33" t="s">
+        <v>116</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I22" s="11"/>
     </row>
@@ -2419,12 +2481,12 @@
         <v>10</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="D23" s="30" t="n">
+        <v>127</v>
+      </c>
+      <c r="D23" s="33" t="n">
         <v>1</v>
       </c>
       <c r="E23" s="21" t="n">
@@ -2433,11 +2495,11 @@
       <c r="F23" s="21" t="n">
         <v>15</v>
       </c>
-      <c r="G23" s="30" t="s">
-        <v>112</v>
+      <c r="G23" s="33" t="s">
+        <v>116</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I23" s="11"/>
     </row>
@@ -2446,12 +2508,12 @@
         <v>10</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="D24" s="30" t="n">
+        <v>128</v>
+      </c>
+      <c r="D24" s="33" t="n">
         <v>1</v>
       </c>
       <c r="E24" s="21" t="n">
@@ -2460,11 +2522,11 @@
       <c r="F24" s="21" t="n">
         <v>10.25</v>
       </c>
-      <c r="G24" s="30" t="s">
-        <v>112</v>
+      <c r="G24" s="33" t="s">
+        <v>116</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I24" s="11"/>
     </row>
@@ -2473,24 +2535,24 @@
         <v>10</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="D25" s="30"/>
-      <c r="E25" s="30"/>
+        <v>129</v>
+      </c>
+      <c r="D25" s="33"/>
+      <c r="E25" s="33"/>
       <c r="F25" s="21" t="n">
         <v>5371.5</v>
       </c>
-      <c r="G25" s="30" t="s">
-        <v>89</v>
+      <c r="G25" s="33" t="s">
+        <v>93</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2498,24 +2560,24 @@
         <v>16</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="D26" s="30"/>
-      <c r="E26" s="30"/>
+        <v>132</v>
+      </c>
+      <c r="D26" s="33"/>
+      <c r="E26" s="33"/>
       <c r="F26" s="21" t="n">
         <v>5000</v>
       </c>
-      <c r="G26" s="30" t="s">
+      <c r="G26" s="33" t="s">
         <v>17</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2526,30 +2588,30 @@
         <v>14</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>131</v>
-      </c>
-      <c r="D27" s="30"/>
-      <c r="E27" s="30"/>
+        <v>135</v>
+      </c>
+      <c r="D27" s="33"/>
+      <c r="E27" s="33"/>
       <c r="F27" s="21" t="n">
         <v>250</v>
       </c>
-      <c r="G27" s="30" t="s">
-        <v>127</v>
+      <c r="G27" s="33" t="s">
+        <v>131</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C28" s="31" t="s">
-        <v>134</v>
-      </c>
-      <c r="F28" s="32" t="n">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C28" s="34" t="s">
+        <v>138</v>
+      </c>
+      <c r="F28" s="35" t="n">
         <f aca="false">SUM(F5:F27)</f>
-        <v>67388.99</v>
+        <v>67578.99</v>
       </c>
     </row>
   </sheetData>
@@ -2582,17 +2644,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>3</v>
@@ -2601,26 +2663,26 @@
         <v>4</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="33" t="n">
+      <c r="A5" s="36" t="n">
         <v>46212</v>
       </c>
       <c r="B5" s="8" t="s">
@@ -2630,113 +2692,113 @@
         <v>11</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="F5" s="21" t="n">
         <v>32228.99</v>
       </c>
-      <c r="G5" s="33" t="n">
+      <c r="G5" s="36" t="n">
         <v>46212</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="33" t="n">
+      <c r="A6" s="36" t="n">
         <v>46223</v>
       </c>
       <c r="B6" s="8" t="s">
         <v>23</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="F6" s="21" t="n">
         <v>311.98</v>
       </c>
-      <c r="G6" s="33" t="n">
+      <c r="G6" s="36" t="n">
         <v>46223</v>
       </c>
       <c r="H6" s="20" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="33" t="n">
+      <c r="A7" s="36" t="n">
         <v>46223</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>19</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="F7" s="21" t="n">
         <v>111.71</v>
       </c>
-      <c r="G7" s="33" t="n">
+      <c r="G7" s="36" t="n">
         <v>46223</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="33" t="n">
+      <c r="A8" s="36" t="n">
         <v>46223</v>
       </c>
       <c r="B8" s="8" t="s">
         <v>19</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F8" s="21" t="n">
         <v>937.5</v>
       </c>
-      <c r="G8" s="33" t="n">
+      <c r="G8" s="36" t="n">
         <v>46223</v>
       </c>
       <c r="H8" s="20" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="33" t="n">
+      <c r="A9" s="36" t="n">
         <v>46227</v>
       </c>
       <c r="B9" s="8" t="s">
@@ -2746,235 +2808,253 @@
         <v>14</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="F9" s="21" t="n">
         <v>3088.3</v>
       </c>
-      <c r="G9" s="33" t="n">
+      <c r="G9" s="36" t="n">
         <v>46227</v>
       </c>
       <c r="H9" s="20" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="33" t="n">
+      <c r="A10" s="36" t="n">
         <v>46225</v>
       </c>
       <c r="B10" s="8" t="s">
         <v>23</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="F10" s="21" t="n">
         <v>162.96</v>
       </c>
-      <c r="G10" s="33" t="n">
+      <c r="G10" s="36" t="n">
         <v>46225</v>
       </c>
       <c r="H10" s="20" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="33" t="n">
+      <c r="A11" s="36" t="n">
         <v>46238</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>23</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="F11" s="21" t="n">
         <v>148.53</v>
       </c>
-      <c r="G11" s="33" t="n">
+      <c r="G11" s="36" t="n">
         <v>46238</v>
       </c>
       <c r="H11" s="20" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="34"/>
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="35"/>
-      <c r="F12" s="36"/>
-      <c r="G12" s="34"/>
-      <c r="H12" s="35"/>
-      <c r="I12" s="35"/>
+      <c r="A12" s="36" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="F12" s="21" t="n">
+        <v>1710</v>
+      </c>
+      <c r="G12" s="36" t="n">
+        <v>46241</v>
+      </c>
+      <c r="H12" s="20" t="s">
+        <v>159</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="34"/>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
-      <c r="F13" s="36"/>
-      <c r="G13" s="34"/>
-      <c r="H13" s="35"/>
-      <c r="I13" s="35"/>
+      <c r="A13" s="37"/>
+      <c r="B13" s="38"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="39"/>
+      <c r="G13" s="37"/>
+      <c r="H13" s="38"/>
+      <c r="I13" s="38"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="34"/>
-      <c r="B14" s="35"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="35"/>
-      <c r="F14" s="36"/>
-      <c r="G14" s="34"/>
-      <c r="H14" s="35"/>
-      <c r="I14" s="35"/>
+      <c r="A14" s="37"/>
+      <c r="B14" s="38"/>
+      <c r="C14" s="38"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="39"/>
+      <c r="G14" s="37"/>
+      <c r="H14" s="38"/>
+      <c r="I14" s="38"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="34"/>
-      <c r="B15" s="35"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="36"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="35"/>
-      <c r="I15" s="35"/>
+      <c r="A15" s="37"/>
+      <c r="B15" s="38"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="37"/>
+      <c r="H15" s="38"/>
+      <c r="I15" s="38"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="34"/>
-      <c r="B16" s="35"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="36"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="35"/>
-      <c r="I16" s="35"/>
+      <c r="A16" s="37"/>
+      <c r="B16" s="38"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="39"/>
+      <c r="G16" s="37"/>
+      <c r="H16" s="38"/>
+      <c r="I16" s="38"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="34"/>
-      <c r="B17" s="35"/>
-      <c r="C17" s="35"/>
-      <c r="D17" s="35"/>
-      <c r="E17" s="35"/>
-      <c r="F17" s="36"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="35"/>
-      <c r="I17" s="35"/>
+      <c r="A17" s="37"/>
+      <c r="B17" s="38"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="38"/>
+      <c r="F17" s="39"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="38"/>
+      <c r="I17" s="38"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="34"/>
-      <c r="B18" s="35"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="35"/>
-      <c r="F18" s="36"/>
-      <c r="G18" s="34"/>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35"/>
+      <c r="A18" s="37"/>
+      <c r="B18" s="38"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="39"/>
+      <c r="G18" s="37"/>
+      <c r="H18" s="38"/>
+      <c r="I18" s="38"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="34"/>
-      <c r="B19" s="35"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="35"/>
-      <c r="F19" s="36"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="35"/>
-      <c r="I19" s="35"/>
+      <c r="A19" s="37"/>
+      <c r="B19" s="38"/>
+      <c r="C19" s="38"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="38"/>
+      <c r="F19" s="39"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="38"/>
+      <c r="I19" s="38"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="34"/>
-      <c r="B20" s="35"/>
-      <c r="C20" s="35"/>
-      <c r="D20" s="35"/>
-      <c r="E20" s="35"/>
-      <c r="F20" s="36"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="35"/>
-      <c r="I20" s="35"/>
+      <c r="A20" s="37"/>
+      <c r="B20" s="38"/>
+      <c r="C20" s="38"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="38"/>
+      <c r="F20" s="39"/>
+      <c r="G20" s="37"/>
+      <c r="H20" s="38"/>
+      <c r="I20" s="38"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="34"/>
-      <c r="B21" s="35"/>
-      <c r="C21" s="35"/>
-      <c r="D21" s="35"/>
-      <c r="E21" s="35"/>
-      <c r="F21" s="36"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="35"/>
-      <c r="I21" s="35"/>
+      <c r="A21" s="37"/>
+      <c r="B21" s="38"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="38"/>
+      <c r="F21" s="39"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="38"/>
+      <c r="I21" s="38"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="34"/>
-      <c r="B22" s="35"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="35"/>
-      <c r="I22" s="35"/>
+      <c r="A22" s="37"/>
+      <c r="B22" s="38"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="39"/>
+      <c r="G22" s="37"/>
+      <c r="H22" s="38"/>
+      <c r="I22" s="38"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="34"/>
-      <c r="B23" s="35"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="35"/>
-      <c r="E23" s="35"/>
-      <c r="F23" s="36"/>
-      <c r="G23" s="34"/>
-      <c r="H23" s="35"/>
-      <c r="I23" s="35"/>
+      <c r="A23" s="37"/>
+      <c r="B23" s="38"/>
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="38"/>
+      <c r="F23" s="39"/>
+      <c r="G23" s="37"/>
+      <c r="H23" s="38"/>
+      <c r="I23" s="38"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="34"/>
-      <c r="B24" s="35"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="34"/>
-      <c r="H24" s="35"/>
-      <c r="I24" s="35"/>
+      <c r="A24" s="37"/>
+      <c r="B24" s="38"/>
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="38"/>
+      <c r="F24" s="39"/>
+      <c r="G24" s="37"/>
+      <c r="H24" s="38"/>
+      <c r="I24" s="38"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="34"/>
-      <c r="B25" s="35"/>
-      <c r="C25" s="35"/>
-      <c r="D25" s="35"/>
-      <c r="E25" s="35"/>
-      <c r="F25" s="36"/>
-      <c r="G25" s="34"/>
-      <c r="H25" s="35"/>
-      <c r="I25" s="35"/>
+      <c r="A25" s="37"/>
+      <c r="B25" s="38"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="39"/>
+      <c r="G25" s="37"/>
+      <c r="H25" s="38"/>
+      <c r="I25" s="38"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3005,61 +3085,61 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="B4" s="37" t="n">
+        <v>177</v>
+      </c>
+      <c r="B4" s="40" t="n">
         <v>1130</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="D4" s="38" t="n">
+        <v>178</v>
+      </c>
+      <c r="D4" s="41" t="n">
         <f aca="false">B4-SUM(E8:E40)</f>
         <v>506.53</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="33" t="n">
+      <c r="A8" s="36" t="n">
         <v>46223</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="E8" s="21" t="n">
         <v>311.98</v>
@@ -3070,17 +3150,17 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="33" t="n">
+      <c r="A9" s="36" t="n">
         <v>46225</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="E9" s="21" t="n">
         <v>162.96</v>
@@ -3091,17 +3171,17 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="33" t="n">
+      <c r="A10" s="36" t="n">
         <v>46238</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="E10" s="21" t="n">
         <v>148.53</v>
@@ -3112,165 +3192,165 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="34"/>
-      <c r="B11" s="35"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="36"/>
+      <c r="A11" s="37"/>
+      <c r="B11" s="38"/>
+      <c r="C11" s="38"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="39"/>
       <c r="F11" s="10" t="str">
         <f aca="false">IF(E11="","",$B$4-SUM($E$8:E11))</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="34"/>
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="36"/>
+      <c r="A12" s="37"/>
+      <c r="B12" s="38"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="39"/>
       <c r="F12" s="10" t="str">
         <f aca="false">IF(E12="","",$B$4-SUM($E$8:E12))</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="34"/>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="36"/>
+      <c r="A13" s="37"/>
+      <c r="B13" s="38"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="39"/>
       <c r="F13" s="10" t="str">
         <f aca="false">IF(E13="","",$B$4-SUM($E$8:E13))</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="34"/>
-      <c r="B14" s="35"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="36"/>
+      <c r="A14" s="37"/>
+      <c r="B14" s="38"/>
+      <c r="C14" s="38"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="39"/>
       <c r="F14" s="10" t="str">
         <f aca="false">IF(E14="","",$B$4-SUM($E$8:E14))</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="34"/>
-      <c r="B15" s="35"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="36"/>
+      <c r="A15" s="37"/>
+      <c r="B15" s="38"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="39"/>
       <c r="F15" s="10" t="str">
         <f aca="false">IF(E15="","",$B$4-SUM($E$8:E15))</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="34"/>
-      <c r="B16" s="35"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="36"/>
+      <c r="A16" s="37"/>
+      <c r="B16" s="38"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="39"/>
       <c r="F16" s="10" t="str">
         <f aca="false">IF(E16="","",$B$4-SUM($E$8:E16))</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="34"/>
-      <c r="B17" s="35"/>
-      <c r="C17" s="35"/>
-      <c r="D17" s="35"/>
-      <c r="E17" s="36"/>
+      <c r="A17" s="37"/>
+      <c r="B17" s="38"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="39"/>
       <c r="F17" s="10" t="str">
         <f aca="false">IF(E17="","",$B$4-SUM($E$8:E17))</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="34"/>
-      <c r="B18" s="35"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="36"/>
+      <c r="A18" s="37"/>
+      <c r="B18" s="38"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="39"/>
       <c r="F18" s="10" t="str">
         <f aca="false">IF(E18="","",$B$4-SUM($E$8:E18))</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="34"/>
-      <c r="B19" s="35"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="36"/>
+      <c r="A19" s="37"/>
+      <c r="B19" s="38"/>
+      <c r="C19" s="38"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="39"/>
       <c r="F19" s="10" t="str">
         <f aca="false">IF(E19="","",$B$4-SUM($E$8:E19))</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="34"/>
-      <c r="B20" s="35"/>
-      <c r="C20" s="35"/>
-      <c r="D20" s="35"/>
-      <c r="E20" s="36"/>
+      <c r="A20" s="37"/>
+      <c r="B20" s="38"/>
+      <c r="C20" s="38"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="39"/>
       <c r="F20" s="10" t="str">
         <f aca="false">IF(E20="","",$B$4-SUM($E$8:E20))</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="34"/>
-      <c r="B21" s="35"/>
-      <c r="C21" s="35"/>
-      <c r="D21" s="35"/>
-      <c r="E21" s="36"/>
+      <c r="A21" s="37"/>
+      <c r="B21" s="38"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="39"/>
       <c r="F21" s="10" t="str">
         <f aca="false">IF(E21="","",$B$4-SUM($E$8:E21))</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="34"/>
-      <c r="B22" s="35"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="36"/>
+      <c r="A22" s="37"/>
+      <c r="B22" s="38"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="39"/>
       <c r="F22" s="10" t="str">
         <f aca="false">IF(E22="","",$B$4-SUM($E$8:E22))</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="34"/>
-      <c r="B23" s="35"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="35"/>
-      <c r="E23" s="36"/>
+      <c r="A23" s="37"/>
+      <c r="B23" s="38"/>
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="39"/>
       <c r="F23" s="10" t="str">
         <f aca="false">IF(E23="","",$B$4-SUM($E$8:E23))</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="34"/>
-      <c r="B24" s="35"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="36"/>
+      <c r="A24" s="37"/>
+      <c r="B24" s="38"/>
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="39"/>
       <c r="F24" s="10" t="str">
         <f aca="false">IF(E24="","",$B$4-SUM($E$8:E24))</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="34"/>
-      <c r="B25" s="35"/>
-      <c r="C25" s="35"/>
-      <c r="D25" s="35"/>
-      <c r="E25" s="36"/>
+      <c r="A25" s="37"/>
+      <c r="B25" s="38"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="39"/>
       <c r="F25" s="10" t="str">
         <f aca="false">IF(E25="","",$B$4-SUM($E$8:E25))</f>
         <v/>
@@ -3303,221 +3383,221 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="B4" s="37" t="n">
+        <v>193</v>
+      </c>
+      <c r="B4" s="40" t="n">
         <v>5000</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="D4" s="38" t="n">
+        <v>178</v>
+      </c>
+      <c r="D4" s="41" t="n">
         <f aca="false">B4-SUM(D8:D40)</f>
         <v>5000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="34"/>
-      <c r="B8" s="35"/>
-      <c r="C8" s="35"/>
-      <c r="D8" s="36"/>
+      <c r="A8" s="37"/>
+      <c r="B8" s="38"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="39"/>
       <c r="E8" s="10" t="str">
         <f aca="false">IF(D8="","",$B$4-SUM($D$8:D8))</f>
         <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="34"/>
-      <c r="B9" s="35"/>
-      <c r="C9" s="35"/>
-      <c r="D9" s="36"/>
+      <c r="A9" s="37"/>
+      <c r="B9" s="38"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="39"/>
       <c r="E9" s="10" t="str">
         <f aca="false">IF(D9="","",$B$4-SUM($D$8:D9))</f>
         <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="34"/>
-      <c r="B10" s="35"/>
-      <c r="C10" s="35"/>
-      <c r="D10" s="36"/>
+      <c r="A10" s="37"/>
+      <c r="B10" s="38"/>
+      <c r="C10" s="38"/>
+      <c r="D10" s="39"/>
       <c r="E10" s="10" t="str">
         <f aca="false">IF(D10="","",$B$4-SUM($D$8:D10))</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="34"/>
-      <c r="B11" s="35"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="36"/>
+      <c r="A11" s="37"/>
+      <c r="B11" s="38"/>
+      <c r="C11" s="38"/>
+      <c r="D11" s="39"/>
       <c r="E11" s="10" t="str">
         <f aca="false">IF(D11="","",$B$4-SUM($D$8:D11))</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="34"/>
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="36"/>
+      <c r="A12" s="37"/>
+      <c r="B12" s="38"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="39"/>
       <c r="E12" s="10" t="str">
         <f aca="false">IF(D12="","",$B$4-SUM($D$8:D12))</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="34"/>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="36"/>
+      <c r="A13" s="37"/>
+      <c r="B13" s="38"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="39"/>
       <c r="E13" s="10" t="str">
         <f aca="false">IF(D13="","",$B$4-SUM($D$8:D13))</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="34"/>
-      <c r="B14" s="35"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="36"/>
+      <c r="A14" s="37"/>
+      <c r="B14" s="38"/>
+      <c r="C14" s="38"/>
+      <c r="D14" s="39"/>
       <c r="E14" s="10" t="str">
         <f aca="false">IF(D14="","",$B$4-SUM($D$8:D14))</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="34"/>
-      <c r="B15" s="35"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="36"/>
+      <c r="A15" s="37"/>
+      <c r="B15" s="38"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="39"/>
       <c r="E15" s="10" t="str">
         <f aca="false">IF(D15="","",$B$4-SUM($D$8:D15))</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="34"/>
-      <c r="B16" s="35"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="36"/>
+      <c r="A16" s="37"/>
+      <c r="B16" s="38"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="39"/>
       <c r="E16" s="10" t="str">
         <f aca="false">IF(D16="","",$B$4-SUM($D$8:D16))</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="34"/>
-      <c r="B17" s="35"/>
-      <c r="C17" s="35"/>
-      <c r="D17" s="36"/>
+      <c r="A17" s="37"/>
+      <c r="B17" s="38"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="39"/>
       <c r="E17" s="10" t="str">
         <f aca="false">IF(D17="","",$B$4-SUM($D$8:D17))</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="34"/>
-      <c r="B18" s="35"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="36"/>
+      <c r="A18" s="37"/>
+      <c r="B18" s="38"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="39"/>
       <c r="E18" s="10" t="str">
         <f aca="false">IF(D18="","",$B$4-SUM($D$8:D18))</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="34"/>
-      <c r="B19" s="35"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="36"/>
+      <c r="A19" s="37"/>
+      <c r="B19" s="38"/>
+      <c r="C19" s="38"/>
+      <c r="D19" s="39"/>
       <c r="E19" s="10" t="str">
         <f aca="false">IF(D19="","",$B$4-SUM($D$8:D19))</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="34"/>
-      <c r="B20" s="35"/>
-      <c r="C20" s="35"/>
-      <c r="D20" s="36"/>
+      <c r="A20" s="37"/>
+      <c r="B20" s="38"/>
+      <c r="C20" s="38"/>
+      <c r="D20" s="39"/>
       <c r="E20" s="10" t="str">
         <f aca="false">IF(D20="","",$B$4-SUM($D$8:D20))</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="34"/>
-      <c r="B21" s="35"/>
-      <c r="C21" s="35"/>
-      <c r="D21" s="36"/>
+      <c r="A21" s="37"/>
+      <c r="B21" s="38"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="39"/>
       <c r="E21" s="10" t="str">
         <f aca="false">IF(D21="","",$B$4-SUM($D$8:D21))</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="34"/>
-      <c r="B22" s="35"/>
-      <c r="C22" s="35"/>
-      <c r="D22" s="36"/>
+      <c r="A22" s="37"/>
+      <c r="B22" s="38"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="39"/>
       <c r="E22" s="10" t="str">
         <f aca="false">IF(D22="","",$B$4-SUM($D$8:D22))</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="34"/>
-      <c r="B23" s="35"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="36"/>
+      <c r="A23" s="37"/>
+      <c r="B23" s="38"/>
+      <c r="C23" s="38"/>
+      <c r="D23" s="39"/>
       <c r="E23" s="10" t="str">
         <f aca="false">IF(D23="","",$B$4-SUM($D$8:D23))</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="34"/>
-      <c r="B24" s="35"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="36"/>
+      <c r="A24" s="37"/>
+      <c r="B24" s="38"/>
+      <c r="C24" s="38"/>
+      <c r="D24" s="39"/>
       <c r="E24" s="10" t="str">
         <f aca="false">IF(D24="","",$B$4-SUM($D$8:D24))</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="34"/>
-      <c r="B25" s="35"/>
-      <c r="C25" s="35"/>
-      <c r="D25" s="36"/>
+      <c r="A25" s="37"/>
+      <c r="B25" s="38"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="39"/>
       <c r="E25" s="10" t="str">
         <f aca="false">IF(D25="","",$B$4-SUM($D$8:D25))</f>
         <v/>

</xml_diff>

<commit_message>
Updates to timeline and tracker
</commit_message>
<xml_diff>
--- a/files/Spinney_Budget_Tracker_v4.xlsx
+++ b/files/Spinney_Budget_Tracker_v4.xlsx
@@ -12,8 +12,9 @@
     <sheet name="Invoicing Schedule" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Cost Lines" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Invoice Register" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Materials Receipts" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Contingency Drawdown" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Skip Hire Log" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Materials Receipts" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Contingency Drawdown" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="223">
   <si>
     <t xml:space="preserve">Spinney External Works — Budget Summary</t>
   </si>
@@ -72,7 +73,7 @@
     <t xml:space="preserve">LG Building and Roofing Ltd</t>
   </si>
   <si>
-    <t xml:space="preserve">£17,600 labour (no VAT) + £1,200 rubbish removal. RISK: price 'fairly accurate' pending Luke's structure/ground assessment.</t>
+    <t xml:space="preserve">Labour £17,600 (no VAT). EXCLUDED from 10% discount. Rubbish removal (£1,200) transferred 10 Aug to pooled skip fund.</t>
   </si>
   <si>
     <t xml:space="preserve">Contingency</t>
@@ -87,13 +88,13 @@
     <t xml:space="preserve">Chimney repair</t>
   </si>
   <si>
-    <t xml:space="preserve">Quoted separately (2 Jun). Labour £3,200 no VAT (invoiced 24 Jul, full price — no cash discount) + £80 rubbish (outstanding) + scaffolding £1,500 share of combined invoice. Materials in pooled budget.</t>
+    <t xml:space="preserve">Quoted separately (2 Jun). Labour £3,200 no VAT (invoiced 24 Jul, full price) + scaffolding £1,500 share + £62.90 additional material (stainless steel cowl, paid 10 Aug). Rubbish removal transferred to pooled skip fund. Materials in pooled budget.</t>
   </si>
   <si>
     <t xml:space="preserve">Coping stones repair</t>
   </si>
   <si>
-    <t xml:space="preserve">Quoted separately (3 Jun). Base labour blended, confirmed 7 Aug: 50% cash (10% disc.) + 50% invoiced = £3610.00. +£80 rubbish (full price, rides with invoice portion). +£1,700 scaffold share. +£250 condensation-prep addition — PRICE NOT FINALISED, terms will be 100% cash + materials, separate from this split. RISK: coping-stone damage on removal could substantially increase cost. Materials in pooled budget.</t>
+    <t xml:space="preserve">Quoted separately (3 Jun). Base labour blended, confirmed 7 Aug: 50% cash (10% disc.) + 50% invoiced = £3,610.00. +£1,700 scaffold share. +£250 condensation-prep addition — PRICE NOT FINALISED. Rubbish removal transferred to pooled skip fund. RISK: coping-stone damage on removal could substantially increase cost. Materials in pooled budget.</t>
   </si>
   <si>
     <t xml:space="preserve">Materials (pooled)</t>
@@ -105,6 +106,15 @@
     <t xml:space="preserve">Pooled chimney (£480) + coping (£650) materials budget — decision 20 Jul. Purchased via merchant trade accounts (Dry Lining Supplies, Travis Perkins etc.), cleared on receipts. Detail on Materials Receipts sheet.</t>
   </si>
   <si>
+    <t xml:space="preserve">Rubbish removal (pooled skips)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skip Hire Comparison Ltd / future providers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transferred 10 Aug from chimney/coping/decking rubbish-removal quotes (£80+£80+£1,200). Provisional — more skips expected, especially during decking. Detail on Skip Hire Log sheet.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Core project (Luke's ~£56,800 outline)</t>
   </si>
   <si>
@@ -144,189 +154,195 @@
     <t xml:space="preserve">Order placed — PAID IN FULL 9 Jul</t>
   </si>
   <si>
-    <t xml:space="preserve">Invoice V4FQ-15584 (Register row 1)</t>
+    <t xml:space="preserve">Invoice V4FQ-15584</t>
   </si>
   <si>
     <t xml:space="preserve">Paid</t>
   </si>
   <si>
-    <t xml:space="preserve">All-Ashwood + flexible bullnose; 144.9 m²</t>
-  </si>
-  <si>
     <t xml:space="preserve">Chimney + Coping (scaffold)</t>
   </si>
   <si>
     <t xml:space="preserve">Erection complete (17–18 Jul) — PAID</t>
   </si>
   <si>
+    <t xml:space="preserve">Scaffolder (via Trevor)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£2,000 cash (of £3,200 combined)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logged in Register: £937.50 chimney + £1,062.50 coping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strike, after Gate 1 sign-off</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£1,200 cash balance on strike</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agreed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log in Register: £562.50 chimney + £637.50 coping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INVOICED &amp; PAID 24 Jul (non-cash)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£3,200 labour less £111.70 prepaid = £3,088.30. Full price — no discount.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£3,200 labour invoiced &amp; paid 24 Jul (£3,088.30 after £111.70 prepayment deduction). Rubbish removal (£80) transferred 10 Aug to pooled skip fund — no longer owed to Luke.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50% CASH — PAID 7 Aug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50% of base labour (£1,710.00), 10% cash discount. Based on original £3,800 quote only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excludes condensation-prep addition — price not yet finalised (see separate row).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50% INVOICED — due next week</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50% of base labour (£1,900.00) full price. Rubbish removal transferred to pooled skip fund 10 Aug.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved 7 Aug — awaiting invoice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No longer includes rubbish removal — see Rubbish removal (pooled skips) row. Timed after back gutters are complete, alongside base coping labour sign-off.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Additional scope — condensation-escape prep (price TBC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Combined labour + materials, Luke's estimate — price NOT yet finalised</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price TBC — not finalised (7 Aug)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terms confirmed 7 Aug: 100% cash (labour + materials) once priced. Separate from the base coping 50/50 split.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4–5 stages — triggers TBC with Luke/Lara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£17,600 labour total across stages. EXCLUDED from 10% labour discount. Rubbish removal transferred to pooled skip fund.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved 20 Jul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suggested triggers: start / substructure (a) / Gate 2 / substructure (b) / Gate 3 — to be pinned</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Periodic — on receipts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Merchant trade accounts (Dry Lining Supplies, TP etc.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pooled £1,130 budget (chimney £480 + coping £650)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agreed in principle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Log each receipt in Register + Materials Receipts sheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rainy-day tasks 100% on completion; named extras as incurred</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LG Building / merchants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£5,000 pot — fence labour, soakaway fix, garage drainage, curved-deck extras, cement &amp; bricks. Labour at 10% discount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Curved-decking extra labour discount TBC. Each drawdown also on Contingency Drawdown sheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Additional material — stainless steel cowl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">StoveWorldUK (paid direct, project account)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Order #147399, 10 Aug 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5" stainless steel chimney pot hanger cowl — replaces original spec (decision logged 7 Aug), prevents rusting. Arrives Fri 14 Aug — likely last item before scaffold strike.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Periodic — as skips are needed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provisional £1,360 (transferred from chimney/coping/decking rubbish quotes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved 10 Aug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First skip £344.16 paid 10 Aug, delivery 11 Aug. More skips expected during decking — budget is provisional, watch like the materials pool. Log each skip in Register + Skip Hire Log sheet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCHEDULE TOTAL (all rows):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summary tab committed total:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Difference (must be £0.00):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost Lines — every line item from LG estimates and the V4 invoice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source documents: LG chimney estimate 2 Jun 2026 · LG coping estimate 3 Jun 2026 · LG decking estimate 3 Jun 2026 · V4 invoice V4FQ-15584, 9 Jul 2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unit £</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line total £</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payment route</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LG Building</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Labour — remove render, k-rend sealer, base + top coat, render crown, storm-dry cream</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No VAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LG invoice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INVOICED 24 Jul (INV-0286), full price £3,200 less £111.70 prepaid = £3,088.30. Non-cash, so 10% discount does not apply. Rubbish removal £80 outstanding.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Scaffolder (direct)</t>
   </si>
   <si>
-    <t xml:space="preserve">£2,000 in cash (of £3,200 combined)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Logged in Register: £937.50 chimney + £1,062.50 coping (pro-rata of £1,500/£1,700)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strike, after Gate 1 sign-off</t>
-  </si>
-  <si>
-    <t xml:space="preserve">£1,200 cash balance on strike</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agreed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Log in Register: £562.50 chimney + £637.50 coping</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INVOICED &amp; PAID 24 Jul (non-cash)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Full price (invoiced, not cash): £3,200 labour + £80 rubbish = £3,280</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INVOICED &amp; PAID 24 Jul: £3,088.30 (labour less £111.70 prepaid). Rubbish £80 NOT yet invoiced — outstanding, follow up with Luke. Needs a couple more days on his return from holiday (timeline TBC, held for now).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">50% CASH — due today, 7 Aug</t>
-  </si>
-  <si>
-    <t xml:space="preserve">50% of base labour (£1710.00), 10% cash discount applied. Based on original £3,800 quote only.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Due today</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONFIRMED 7 Aug. Excludes condensation-prep addition — its price is not yet finalised (see separate row).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">50% INVOICED — due next week</t>
-  </si>
-  <si>
-    <t xml:space="preserve">50% of base labour (£1900.00) full price, + £80 rubbish removal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Approved 7 Aug — awaiting invoice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rubbish removal assumed to ride with this invoice (unconfirmed — chimney's £80 is still outstanding as a comparator).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Additional scope — condensation-escape prep (price TBC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Combined labour + materials, Luke's estimate — price NOT yet finalised</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Price TBC — not finalised (7 Aug)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Terms confirmed 7 Aug: 100% cash (labour + materials) once priced. Separate from the base coping 50/50 split. £250 is provisional.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4–5 stages — triggers TBC with Luke/Lara</t>
-  </si>
-  <si>
-    <t xml:space="preserve">£18,800 total across stages. EXCLUDED from 10% labour discount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Approved 20 Jul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Suggested triggers: start / substructure (a) / Gate 2 / substructure (b) / Gate 3 — to be pinned</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Periodic — on receipts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Merchant trade accounts (Dry Lining Supplies, TP etc.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pooled £1,130 budget (chimney £480 + coping £650)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agreed in principle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Log each receipt in Register + Materials Receipts sheet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rainy-day tasks 100% on completion; named extras as incurred</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LG Building / merchants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">£5,000 pot — fence labour, soakaway fix, garage drainage, curved-deck extras, cement &amp; bricks. Labour at 10% discount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Curved-decking extra labour discount TBC (decking exclusion boundary). Each drawdown also on Contingency Drawdown sheet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCHEDULE TOTAL (all rows):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pooled £1,130 budget — log each receipt in Register + Materials Receipts sheet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rainy-day tasks invoiced 100% on completion; named extras as incurred</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LG Building / Travis Perkins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Summary tab committed total:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rainy-day tasks invoiced 100% on completion, labour less 10%. Curved-decking extra labour discount TBC. Each drawdown also logged on Contingency Drawdown sheet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Difference (must be £0.00):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cost Lines — every line item from LG estimates and the V4 invoice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source documents: LG chimney estimate 2 Jun 2026 · LG coping estimate 3 Jun 2026 · LG decking estimate 3 Jun 2026 · V4 invoice V4FQ-15584, 9 Jul 2026.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Line item</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Qty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unit £</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Line total £</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VAT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Payment route</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LG Building</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Labour — remove render, k-rend sealer, base + top coat, render crown, storm-dry cream</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No VAT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LG invoice</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INVOICED 24 Jul (INV-0286), full price £3,200 less £111.70 prepaid = £3,088.30. Non-cash, so 10% discount does not apply. Rubbish removal £80 outstanding.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tubular scaffolding — all four sides of chimney and crown</t>
   </si>
   <si>
@@ -348,10 +364,13 @@
     <t xml:space="preserve">Rubbish removal</t>
   </si>
   <si>
+    <t xml:space="preserve">TRANSFERRED 10 Aug to pooled Rubbish removal (skips) fund — family now supplies skips directly rather than Luke arranging disposal. No longer owed to Luke.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Labour — remove/reset copings, slate cap, render, lead flashings to parapet rear</t>
   </si>
   <si>
-    <t xml:space="preserve">CONFIRMED 7 Aug, based on original £3,800 quote: 50% cash (£1710.00 @ 10% discount) due same day, 50% invoiced (£1900.00 full price) due next week. RISK: coping-stone damage on removal could substantially increase cost.</t>
+    <t xml:space="preserve">CONFIRMED 7 Aug, based on original £3,800 quote: 50% cash (£1710.00 @ 10% discount) due same day, 50% invoiced (£1900.00 full price) due next week, timed after back gutters are complete — see Invoicing Schedule. RISK: coping-stone damage on removal could substantially increase cost.</t>
   </si>
   <si>
     <t xml:space="preserve">Tubular scaffolding with winch system</t>
@@ -360,6 +379,9 @@
     <t xml:space="preserve">Materials (coping estimate — pooled 20 Jul)</t>
   </si>
   <si>
+    <t xml:space="preserve">TRANSFERRED 10 Aug to pooled Rubbish removal (skips) fund. Removed from next week's invoice (now £1,900, not £1,980).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Labour — remove old decking &amp; frame, construct composite frame, install deck to spec</t>
   </si>
   <si>
@@ -369,6 +391,9 @@
     <t xml:space="preserve">Rubbish removal (8-yard skips ×2, possibly 3)</t>
   </si>
   <si>
+    <t xml:space="preserve">TRANSFERRED 10 Aug to pooled Rubbish removal (skips) fund.</t>
+  </si>
+  <si>
     <t xml:space="preserve">V4 Wood Flooring</t>
   </si>
   <si>
@@ -441,6 +466,24 @@
     <t xml:space="preserve">PRICE NOT YET FINALISED (7 Aug). Terms confirmed: 100% cash (labour + materials) once priced — separate from the base coping 50/50 split. £250 is Luke's original estimate only; treat as provisional until a firm figure is given.</t>
   </si>
   <si>
+    <t xml:space="preserve">StoveWorldUK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Additional material — 5" Stainless Steel Chimney Pot Hanger Cowl (order #147399), replaces original spec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid direct by Ryan (project account)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decision logged 7 Aug (stainless steel, prevent rusting). Cost finalised 10 Aug. Arrives Fri 14 Aug — likely last item before scaffold strike.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provisional pooled budget — transferred from chimney (£80) + coping (£80) + decking (£1,200) rubbish-removal quotes, 10 Aug. Family now supplies skips directly.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First skip ordered 10 Aug (£344.16, 8yd, delivery 11 Aug). More skips expected during decking — budget is provisional, to be watched like the materials pool. Detail on Skip Hire Log sheet.</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOTAL (all lines)</t>
   </si>
   <si>
@@ -501,9 +544,6 @@
     <t xml:space="preserve">PREPAYMENT vs chimney phase-start invoice: pay £1,528.29 of the £1,640 when it lands</t>
   </si>
   <si>
-    <t xml:space="preserve">Scaffolder (via Trevor)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Cash</t>
   </si>
   <si>
@@ -552,34 +592,76 @@
     <t xml:space="preserve">Confirmed 7 Aug: 50% cash / 50% invoice split on original £3,800 quote. Remainder £1,980.00 (incl. rubbish) to be invoiced next week. £250 addition separate, price TBC.</t>
   </si>
   <si>
+    <t xml:space="preserve">Order #147399</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5" Stainless Steel Chimney Pot Hanger Cowl — replaces original spec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Card (Ryan, project account)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmed decision 7 Aug (stainless steel, prevent rusting). Own line under chimney, not pooled materials — different supplier/route to shared render consumables. Arrives Fri 14 Aug.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skip Hire Comparison Ltd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D81F29CE-0002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 cubic yard skip, delivery 11 Aug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First skip. Replaces chimney/coping/decking rubbish-removal quotes — transferred to this pooled fund 10 Aug.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skip Hire Log — pooled rubbish-removal drawdown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provisional pooled budget £1,360 (transferred 10 Aug from chimney £80 + coping £80 + decking £1,200 rubbish-removal quotes). Family now supplies skips directly rather than Luke arranging disposal. Log every skip here AND on the Invoice Register (cost centre: Rubbish removal (pooled skips)) — this sheet is skip detail, the Register is the money record. Unlike the materials pool, more skips are expected — budget may need topping up.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opening pool:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remaining:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provider</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Skip details</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase / use</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amount £</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Running remaining £</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 cubic yard, general waste, delivery 11 Aug (ref D81F29CE-0002)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Above-ground works (chimney/coping)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Materials Receipts — pooled budget drawdown</t>
   </si>
   <si>
     <t xml:space="preserve">Pooled budget £1,130 (chimney £480 + coping £650, pooled 20 Jul). Log every merchant receipt here AND on the Invoice Register (cost centre: Materials (pooled)) — this sheet is the pool detail, the Register is the money record.</t>
   </si>
   <si>
-    <t xml:space="preserve">Opening pool:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Remaining:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Date</t>
-  </si>
-  <si>
     <t xml:space="preserve">Merchant</t>
   </si>
   <si>
     <t xml:space="preserve">Items (summary)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phase / use</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amount £</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Running remaining £</t>
   </si>
   <si>
     <t xml:space="preserve">Render mesh, Weberend Aid ×6, angle/stop beads, rubble sacks, Bond It SBR 5l (project share; £111.71 platform excluded — Luke's equipment)</t>
@@ -831,7 +913,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="47">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -884,6 +966,26 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -892,7 +994,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -900,11 +1010,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -932,35 +1042,27 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1272,7 +1374,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="n">
-        <v>46241</v>
+        <v>46244</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>2</v>
@@ -1335,7 +1437,7 @@
         <v>14</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>18800</v>
+        <v>17600</v>
       </c>
       <c r="D6" s="10" t="n">
         <f aca="false">SUMIF('Invoice Register'!$B:$B,$A6,'Invoice Register'!$F:$F)</f>
@@ -1347,7 +1449,7 @@
       </c>
       <c r="F6" s="10" t="n">
         <f aca="false">C6-D6</f>
-        <v>18800</v>
+        <v>17600</v>
       </c>
       <c r="G6" s="12" t="s">
         <v>15</v>
@@ -1387,19 +1489,19 @@
         <v>14</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>4780</v>
+        <v>4762.9</v>
       </c>
       <c r="D8" s="10" t="n">
         <f aca="false">SUMIF('Invoice Register'!$B:$B,$A8,'Invoice Register'!$F:$F)</f>
-        <v>4137.51</v>
+        <v>4200.41</v>
       </c>
       <c r="E8" s="10" t="n">
         <f aca="false">SUMIFS('Invoice Register'!$F:$F,'Invoice Register'!$B:$B,$A8,'Invoice Register'!$G:$G,"&lt;&gt;")</f>
-        <v>4137.51</v>
+        <v>4200.41</v>
       </c>
       <c r="F8" s="10" t="n">
         <f aca="false">C8-D8</f>
-        <v>642.49</v>
+        <v>562.49</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>20</v>
@@ -1413,7 +1515,7 @@
         <v>14</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>5640</v>
+        <v>5560</v>
       </c>
       <c r="D9" s="10" t="n">
         <f aca="false">SUMIF('Invoice Register'!$B:$B,$A9,'Invoice Register'!$F:$F)</f>
@@ -1425,7 +1527,7 @@
       </c>
       <c r="F9" s="10" t="n">
         <f aca="false">C9-D9</f>
-        <v>3930</v>
+        <v>3850</v>
       </c>
       <c r="G9" s="12" t="s">
         <v>22</v>
@@ -1461,77 +1563,102 @@
       <c r="A11" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="14"/>
+      <c r="B11" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="C11" s="15" t="n">
+        <v>1360</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <f aca="false">SUMIF('Invoice Register'!$B:$B,$A11,'Invoice Register'!$F:$F)</f>
+        <v>344.16</v>
+      </c>
+      <c r="E11" s="16" t="n">
+        <f aca="false">SUMIFS('Invoice Register'!$F:$F,'Invoice Register'!$B:$B,$A11,'Invoice Register'!$G:$G,"&lt;&gt;")</f>
+        <v>344.16</v>
+      </c>
+      <c r="F11" s="16" t="n">
+        <f aca="false">C11-D11</f>
+        <v>1015.84</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="B12" s="19"/>
+      <c r="C12" s="15" t="n">
         <f aca="false">C5+C6+C7</f>
-        <v>56028.99</v>
-      </c>
-      <c r="D11" s="15" t="n">
+        <v>54828.99</v>
+      </c>
+      <c r="D12" s="15" t="n">
         <f aca="false">D5+D6+D7</f>
         <v>32228.99</v>
       </c>
-      <c r="E11" s="15" t="n">
+      <c r="E12" s="15" t="n">
         <f aca="false">E5+E6+E7</f>
         <v>32228.99</v>
       </c>
-      <c r="F11" s="15" t="n">
+      <c r="F12" s="15" t="n">
         <f aca="false">F5+F6+F7</f>
-        <v>23800</v>
-      </c>
-      <c r="G11" s="14"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="15" t="n">
+        <v>22600</v>
+      </c>
+      <c r="G12" s="19"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="21"/>
+      <c r="C13" s="22" t="n">
         <f aca="false">C8+C9+C10</f>
-        <v>11550</v>
-      </c>
-      <c r="D12" s="15" t="n">
+        <v>11452.9</v>
+      </c>
+      <c r="D13" s="22" t="n">
         <f aca="false">D8+D9+D10</f>
-        <v>6470.98</v>
-      </c>
-      <c r="E12" s="15" t="n">
+        <v>6533.88</v>
+      </c>
+      <c r="E13" s="22" t="n">
         <f aca="false">E8+E9+E10</f>
-        <v>6470.98</v>
-      </c>
-      <c r="F12" s="15" t="n">
+        <v>6533.88</v>
+      </c>
+      <c r="F13" s="22" t="n">
         <f aca="false">F8+F9+F10</f>
-        <v>5079.02</v>
-      </c>
-      <c r="G12" s="14"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="17"/>
-      <c r="C13" s="18" t="n">
-        <f aca="false">C11+C12</f>
-        <v>67578.99</v>
-      </c>
-      <c r="D13" s="18" t="n">
-        <f aca="false">D11+D12</f>
-        <v>38699.97</v>
-      </c>
-      <c r="E13" s="18" t="n">
-        <f aca="false">E11+E12</f>
-        <v>38699.97</v>
-      </c>
-      <c r="F13" s="18" t="n">
-        <f aca="false">F11+F12</f>
-        <v>28879.02</v>
-      </c>
-      <c r="G13" s="17"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+        <v>4919.02</v>
+      </c>
+      <c r="G13" s="21"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="23" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="24"/>
+      <c r="C14" s="25" t="n">
+        <f aca="false">C11+C12+C13</f>
+        <v>67641.89</v>
+      </c>
+      <c r="D14" s="25" t="n">
+        <f aca="false">D11+D12+D13</f>
+        <v>39107.03</v>
+      </c>
+      <c r="E14" s="25" t="n">
+        <f aca="false">E11+E12+E13</f>
+        <v>39107.03</v>
+      </c>
+      <c r="F14" s="25" t="n">
+        <f aca="false">F11+F12+F13</f>
+        <v>28534.86</v>
+      </c>
+      <c r="G14" s="24"/>
+    </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B15" s="19" t="n">
+        <v>32</v>
+      </c>
+      <c r="B15" s="26" t="n">
         <f aca="false">'Contingency Drawdown'!$D$4</f>
         <v>5000</v>
       </c>
@@ -1552,7 +1679,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
@@ -1566,199 +1693,197 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="H4" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="n">
+      <c r="A5" s="27" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>10</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>11</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="F5" s="21" t="n">
+        <v>42</v>
+      </c>
+      <c r="F5" s="28" t="n">
         <v>32228.99</v>
       </c>
-      <c r="G5" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="H5" s="8" t="s">
-        <v>41</v>
-      </c>
+      <c r="G5" s="29" t="s">
+        <v>43</v>
+      </c>
+      <c r="H5" s="8"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="n">
+      <c r="A6" s="27" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C6" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F6" s="28" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G6" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="H6" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="E6" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F6" s="21" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G6" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="H6" s="8" t="s">
+      <c r="C7" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>44</v>
-      </c>
       <c r="E7" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F7" s="21" t="n">
+        <v>50</v>
+      </c>
+      <c r="F7" s="28" t="n">
         <v>1200</v>
       </c>
-      <c r="G7" s="23" t="s">
-        <v>49</v>
+      <c r="G7" s="30" t="s">
+        <v>51</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20" t="n">
+      <c r="A8" s="27" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="8" t="s">
         <v>19</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>14</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="F8" s="21" t="n">
-        <v>3280</v>
-      </c>
-      <c r="G8" s="22" t="s">
-        <v>40</v>
+        <v>54</v>
+      </c>
+      <c r="F8" s="28" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G8" s="29" t="s">
+        <v>43</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="n">
+      <c r="A9" s="27" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="8" t="s">
         <v>21</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>14</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="F9" s="21" t="n">
+        <v>57</v>
+      </c>
+      <c r="F9" s="28" t="n">
         <v>1710</v>
       </c>
-      <c r="G9" s="24" t="s">
-        <v>56</v>
+      <c r="G9" s="29" t="s">
+        <v>43</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="n">
+      <c r="A10" s="27" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="8" t="s">
         <v>21</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>14</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="F10" s="21" t="n">
-        <v>1980</v>
-      </c>
-      <c r="G10" s="24" t="s">
         <v>60</v>
       </c>
+      <c r="F10" s="28" t="n">
+        <v>1900</v>
+      </c>
+      <c r="G10" s="30" t="s">
+        <v>61</v>
+      </c>
       <c r="H10" s="8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
-        <v>62</v>
+      <c r="A11" s="27" t="n">
+        <v>7</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>21</v>
@@ -1772,10 +1897,10 @@
       <c r="E11" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F11" s="21" t="n">
+      <c r="F11" s="28" t="n">
         <v>250</v>
       </c>
-      <c r="G11" s="24" t="s">
+      <c r="G11" s="31" t="s">
         <v>65</v>
       </c>
       <c r="H11" s="8" t="s">
@@ -1783,8 +1908,8 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20" t="n">
-        <v>6</v>
+      <c r="A12" s="27" t="n">
+        <v>8</v>
       </c>
       <c r="B12" s="8" t="s">
         <v>13</v>
@@ -1798,10 +1923,10 @@
       <c r="E12" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="F12" s="21" t="n">
-        <v>18800</v>
-      </c>
-      <c r="G12" s="23" t="s">
+      <c r="F12" s="28" t="n">
+        <v>17600</v>
+      </c>
+      <c r="G12" s="30" t="s">
         <v>69</v>
       </c>
       <c r="H12" s="8" t="s">
@@ -1809,8 +1934,8 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="n">
-        <v>7</v>
+      <c r="A13" s="27" t="n">
+        <v>9</v>
       </c>
       <c r="B13" s="8" t="s">
         <v>23</v>
@@ -1824,10 +1949,10 @@
       <c r="E13" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="F13" s="21" t="n">
+      <c r="F13" s="28" t="n">
         <v>1130</v>
       </c>
-      <c r="G13" s="23" t="s">
+      <c r="G13" s="30" t="s">
         <v>74</v>
       </c>
       <c r="H13" s="8" t="s">
@@ -1835,8 +1960,8 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="n">
-        <v>8</v>
+      <c r="A14" s="27" t="n">
+        <v>10</v>
       </c>
       <c r="B14" s="8" t="s">
         <v>16</v>
@@ -1850,10 +1975,10 @@
       <c r="E14" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="F14" s="21" t="n">
+      <c r="F14" s="28" t="n">
         <v>5000</v>
       </c>
-      <c r="G14" s="23" t="s">
+      <c r="G14" s="30" t="s">
         <v>69</v>
       </c>
       <c r="H14" s="8" t="s">
@@ -1861,92 +1986,114 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="n">
-        <v>9</v>
+      <c r="A15" s="27" t="n">
+        <v>11</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="E15" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="F15" s="26" t="n">
-        <f aca="false">SUM(F5:F14)</f>
-        <v>67578.99</v>
-      </c>
-      <c r="G15" s="23" t="s">
-        <v>74</v>
+        <v>81</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="F15" s="28" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="G15" s="29" t="s">
+        <v>43</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20" t="n">
-        <v>10</v>
+      <c r="A16" s="27" t="n">
+        <v>11</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="F16" s="27" t="n">
-        <f aca="false">Summary!$C$13</f>
-        <v>67578.99</v>
-      </c>
-      <c r="G16" s="23" t="s">
-        <v>69</v>
+        <v>27</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="F16" s="32" t="n">
+        <v>1360</v>
+      </c>
+      <c r="G16" s="30" t="s">
+        <v>86</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="E17" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="F17" s="28" t="n">
-        <f aca="false">F15-F16</f>
+      <c r="A17" s="33"/>
+      <c r="B17" s="33"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="34" t="s">
+        <v>88</v>
+      </c>
+      <c r="F17" s="35" t="n">
+        <f aca="false">SUM(F5:F16)</f>
+        <v>67641.89</v>
+      </c>
+      <c r="G17" s="33"/>
+      <c r="H17" s="33"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="33"/>
+      <c r="B18" s="33"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="F18" s="37" t="n">
+        <f aca="false">Summary!$C$14</f>
+        <v>67641.89</v>
+      </c>
+      <c r="G18" s="33"/>
+      <c r="H18" s="33"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="33"/>
+      <c r="B19" s="33"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="F19" s="37" t="n">
+        <f aca="false">F17-F18</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="29"/>
-      <c r="B18" s="29"/>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="30" t="s">
-        <v>84</v>
-      </c>
-      <c r="F18" s="31" t="n">
-        <f aca="false">Summary!$C$13</f>
-        <v>67578.99</v>
-      </c>
-      <c r="G18" s="29"/>
-      <c r="H18" s="29"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E19" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="F19" s="32" t="n">
-        <f aca="false">F15-F16</f>
-        <v>0</v>
-      </c>
-    </row>
+      <c r="G19" s="33"/>
+      <c r="H19" s="33"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="33"/>
+      <c r="B20" s="33"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="33"/>
+      <c r="H20" s="33"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1963,7 +2110,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
@@ -1979,12 +2126,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1995,22 +2142,22 @@
         <v>4</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>9</v>
@@ -2021,24 +2168,24 @@
         <v>19</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="28" t="n">
         <v>3200</v>
       </c>
-      <c r="G5" s="33" t="s">
-        <v>97</v>
+      <c r="G5" s="38" t="s">
+        <v>101</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2046,24 +2193,24 @@
         <v>19</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>44</v>
+        <v>104</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="D6" s="33"/>
-      <c r="E6" s="33"/>
-      <c r="F6" s="21" t="n">
+        <v>105</v>
+      </c>
+      <c r="D6" s="38"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="28" t="n">
         <v>1500</v>
       </c>
-      <c r="G6" s="33" t="s">
-        <v>101</v>
+      <c r="G6" s="38" t="s">
+        <v>106</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2074,18 +2221,18 @@
         <v>24</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="D7" s="33"/>
-      <c r="E7" s="33"/>
-      <c r="F7" s="21" t="n">
+        <v>109</v>
+      </c>
+      <c r="D7" s="38"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="28" t="n">
         <v>480</v>
       </c>
-      <c r="G7" s="33" t="s">
-        <v>101</v>
+      <c r="G7" s="38" t="s">
+        <v>106</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="I7" s="11"/>
     </row>
@@ -2094,47 +2241,49 @@
         <v>19</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C8" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="38" t="s">
         <v>106</v>
       </c>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="21" t="n">
-        <v>80</v>
-      </c>
-      <c r="G8" s="33" t="s">
-        <v>101</v>
-      </c>
       <c r="H8" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="I8" s="11"/>
+        <v>102</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
         <v>21</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="D9" s="33"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="21" t="n">
+        <v>113</v>
+      </c>
+      <c r="D9" s="38"/>
+      <c r="E9" s="38"/>
+      <c r="F9" s="28" t="n">
         <v>3610</v>
       </c>
-      <c r="G9" s="33" t="s">
-        <v>97</v>
+      <c r="G9" s="38" t="s">
+        <v>101</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2142,24 +2291,24 @@
         <v>21</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>44</v>
+        <v>104</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="D10" s="33"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="21" t="n">
+        <v>115</v>
+      </c>
+      <c r="D10" s="38"/>
+      <c r="E10" s="38"/>
+      <c r="F10" s="28" t="n">
         <v>1700</v>
       </c>
-      <c r="G10" s="33" t="s">
-        <v>101</v>
+      <c r="G10" s="38" t="s">
+        <v>106</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2170,18 +2319,18 @@
         <v>24</v>
       </c>
       <c r="C11" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="D11" s="38"/>
+      <c r="E11" s="38"/>
+      <c r="F11" s="28" t="n">
+        <v>650</v>
+      </c>
+      <c r="G11" s="38" t="s">
+        <v>106</v>
+      </c>
+      <c r="H11" s="8" t="s">
         <v>110</v>
-      </c>
-      <c r="D11" s="33"/>
-      <c r="E11" s="33"/>
-      <c r="F11" s="21" t="n">
-        <v>650</v>
-      </c>
-      <c r="G11" s="33" t="s">
-        <v>101</v>
-      </c>
-      <c r="H11" s="8" t="s">
-        <v>105</v>
       </c>
       <c r="I11" s="11"/>
     </row>
@@ -2190,47 +2339,49 @@
         <v>21</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C12" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="D12" s="38"/>
+      <c r="E12" s="38"/>
+      <c r="F12" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="38" t="s">
         <v>106</v>
       </c>
-      <c r="D12" s="33"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="21" t="n">
-        <v>80</v>
-      </c>
-      <c r="G12" s="33" t="s">
-        <v>101</v>
-      </c>
       <c r="H12" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="I12" s="11"/>
+        <v>102</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
         <v>13</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="D13" s="33"/>
-      <c r="E13" s="33"/>
-      <c r="F13" s="21" t="n">
+        <v>118</v>
+      </c>
+      <c r="D13" s="38"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="28" t="n">
         <v>17600</v>
       </c>
-      <c r="G13" s="33" t="s">
-        <v>97</v>
+      <c r="G13" s="38" t="s">
+        <v>101</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="I13" s="12" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2238,48 +2389,50 @@
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="D14" s="33"/>
-      <c r="E14" s="33"/>
-      <c r="F14" s="21" t="n">
-        <v>1200</v>
-      </c>
-      <c r="G14" s="33" t="s">
-        <v>101</v>
+        <v>120</v>
+      </c>
+      <c r="D14" s="38"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="38" t="s">
+        <v>106</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="I14" s="11"/>
+        <v>102</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
         <v>10</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="D15" s="33" t="n">
+        <v>123</v>
+      </c>
+      <c r="D15" s="38" t="n">
         <v>230</v>
       </c>
-      <c r="E15" s="21" t="n">
+      <c r="E15" s="28" t="n">
         <v>66.49</v>
       </c>
-      <c r="F15" s="21" t="n">
+      <c r="F15" s="28" t="n">
         <v>15292.7</v>
       </c>
-      <c r="G15" s="33" t="s">
-        <v>116</v>
+      <c r="G15" s="38" t="s">
+        <v>124</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="I15" s="11"/>
     </row>
@@ -2288,25 +2441,25 @@
         <v>10</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="D16" s="33" t="n">
+        <v>126</v>
+      </c>
+      <c r="D16" s="38" t="n">
         <v>18</v>
       </c>
-      <c r="E16" s="21" t="n">
+      <c r="E16" s="28" t="n">
         <v>58.09</v>
       </c>
-      <c r="F16" s="21" t="n">
+      <c r="F16" s="28" t="n">
         <v>1045.62</v>
       </c>
-      <c r="G16" s="33" t="s">
-        <v>116</v>
+      <c r="G16" s="38" t="s">
+        <v>124</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="I16" s="11"/>
     </row>
@@ -2315,28 +2468,28 @@
         <v>10</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="D17" s="33" t="n">
+        <v>127</v>
+      </c>
+      <c r="D17" s="38" t="n">
         <v>15</v>
       </c>
-      <c r="E17" s="21" t="n">
+      <c r="E17" s="28" t="n">
         <v>72.25</v>
       </c>
-      <c r="F17" s="21" t="n">
+      <c r="F17" s="28" t="n">
         <v>1083.75</v>
       </c>
-      <c r="G17" s="33" t="s">
-        <v>116</v>
+      <c r="G17" s="38" t="s">
+        <v>124</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="I17" s="11" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2344,25 +2497,25 @@
         <v>10</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="D18" s="33" t="n">
+        <v>129</v>
+      </c>
+      <c r="D18" s="38" t="n">
         <v>15</v>
       </c>
-      <c r="E18" s="21" t="n">
+      <c r="E18" s="28" t="n">
         <v>59.89</v>
       </c>
-      <c r="F18" s="21" t="n">
+      <c r="F18" s="28" t="n">
         <v>898.35</v>
       </c>
-      <c r="G18" s="33" t="s">
-        <v>116</v>
+      <c r="G18" s="38" t="s">
+        <v>124</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="I18" s="11"/>
     </row>
@@ -2371,25 +2524,25 @@
         <v>10</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>122</v>
-      </c>
-      <c r="D19" s="33" t="n">
+        <v>130</v>
+      </c>
+      <c r="D19" s="38" t="n">
         <v>24</v>
       </c>
-      <c r="E19" s="21" t="n">
+      <c r="E19" s="28" t="n">
         <v>32.08</v>
       </c>
-      <c r="F19" s="21" t="n">
+      <c r="F19" s="28" t="n">
         <v>770</v>
       </c>
-      <c r="G19" s="33" t="s">
-        <v>116</v>
+      <c r="G19" s="38" t="s">
+        <v>124</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="I19" s="11"/>
     </row>
@@ -2398,25 +2551,25 @@
         <v>10</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="D20" s="33" t="n">
+        <v>131</v>
+      </c>
+      <c r="D20" s="38" t="n">
         <v>6</v>
       </c>
-      <c r="E20" s="21" t="n">
+      <c r="E20" s="28" t="n">
         <v>10.25</v>
       </c>
-      <c r="F20" s="21" t="n">
+      <c r="F20" s="28" t="n">
         <v>61.5</v>
       </c>
-      <c r="G20" s="33" t="s">
-        <v>116</v>
+      <c r="G20" s="38" t="s">
+        <v>124</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="I20" s="11"/>
     </row>
@@ -2425,28 +2578,28 @@
         <v>10</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C21" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="D21" s="38" t="n">
+        <v>266</v>
+      </c>
+      <c r="E21" s="28" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="F21" s="28" t="n">
+        <v>7554.4</v>
+      </c>
+      <c r="G21" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="D21" s="33" t="n">
-        <v>266</v>
-      </c>
-      <c r="E21" s="21" t="n">
-        <v>28.4</v>
-      </c>
-      <c r="F21" s="21" t="n">
-        <v>7554.4</v>
-      </c>
-      <c r="G21" s="33" t="s">
-        <v>116</v>
-      </c>
       <c r="H21" s="8" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2454,25 +2607,25 @@
         <v>10</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="D22" s="33" t="n">
+        <v>134</v>
+      </c>
+      <c r="D22" s="38" t="n">
         <v>16</v>
       </c>
-      <c r="E22" s="21" t="n">
+      <c r="E22" s="28" t="n">
         <v>7.87</v>
       </c>
-      <c r="F22" s="21" t="n">
+      <c r="F22" s="28" t="n">
         <v>125.92</v>
       </c>
-      <c r="G22" s="33" t="s">
-        <v>116</v>
+      <c r="G22" s="38" t="s">
+        <v>124</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="I22" s="11"/>
     </row>
@@ -2481,25 +2634,25 @@
         <v>10</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="D23" s="33" t="n">
+        <v>135</v>
+      </c>
+      <c r="D23" s="38" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="21" t="n">
+      <c r="E23" s="28" t="n">
         <v>15</v>
       </c>
-      <c r="F23" s="21" t="n">
+      <c r="F23" s="28" t="n">
         <v>15</v>
       </c>
-      <c r="G23" s="33" t="s">
-        <v>116</v>
+      <c r="G23" s="38" t="s">
+        <v>124</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="I23" s="11"/>
     </row>
@@ -2508,25 +2661,25 @@
         <v>10</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="D24" s="33" t="n">
+        <v>136</v>
+      </c>
+      <c r="D24" s="38" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="21" t="n">
+      <c r="E24" s="28" t="n">
         <v>10.25</v>
       </c>
-      <c r="F24" s="21" t="n">
+      <c r="F24" s="28" t="n">
         <v>10.25</v>
       </c>
-      <c r="G24" s="33" t="s">
-        <v>116</v>
+      <c r="G24" s="38" t="s">
+        <v>124</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="I24" s="11"/>
     </row>
@@ -2535,24 +2688,24 @@
         <v>10</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="D25" s="33"/>
-      <c r="E25" s="33"/>
-      <c r="F25" s="21" t="n">
+        <v>137</v>
+      </c>
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="28" t="n">
         <v>5371.5</v>
       </c>
-      <c r="G25" s="33" t="s">
-        <v>93</v>
+      <c r="G25" s="38" t="s">
+        <v>97</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2560,24 +2713,24 @@
         <v>16</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="D26" s="33"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="21" t="n">
+        <v>140</v>
+      </c>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="28" t="n">
         <v>5000</v>
       </c>
-      <c r="G26" s="33" t="s">
+      <c r="G26" s="38" t="s">
         <v>17</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="I26" s="11" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2588,30 +2741,84 @@
         <v>14</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="D27" s="33"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="21" t="n">
+        <v>143</v>
+      </c>
+      <c r="D27" s="38"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="28" t="n">
         <v>250</v>
       </c>
-      <c r="G27" s="33" t="s">
-        <v>131</v>
+      <c r="G27" s="38" t="s">
+        <v>139</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C28" s="34" t="s">
-        <v>138</v>
-      </c>
-      <c r="F28" s="35" t="n">
-        <f aca="false">SUM(F5:F27)</f>
-        <v>67578.99</v>
+      <c r="A28" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="D28" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="28" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="F28" s="28" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="G28" s="38" t="s">
+        <v>106</v>
+      </c>
+      <c r="H28" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="I28" s="8" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="D29" s="38"/>
+      <c r="E29" s="38"/>
+      <c r="F29" s="28" t="n">
+        <v>1360</v>
+      </c>
+      <c r="G29" s="38" t="s">
+        <v>17</v>
+      </c>
+      <c r="H29" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="I29" s="8" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C30" s="39" t="s">
+        <v>152</v>
+      </c>
+      <c r="F30" s="40" t="n">
+        <f aca="false">SUM(F5:F29)</f>
+        <v>67641.89</v>
       </c>
     </row>
   </sheetData>
@@ -2644,17 +2851,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>3</v>
@@ -2663,26 +2870,26 @@
         <v>4</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>143</v>
+        <v>157</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>145</v>
+        <v>159</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>146</v>
+        <v>160</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="36" t="n">
+      <c r="A5" s="41" t="n">
         <v>46212</v>
       </c>
       <c r="B5" s="8" t="s">
@@ -2692,113 +2899,113 @@
         <v>11</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>147</v>
+        <v>161</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="F5" s="21" t="n">
+        <v>162</v>
+      </c>
+      <c r="F5" s="28" t="n">
         <v>32228.99</v>
       </c>
-      <c r="G5" s="36" t="n">
+      <c r="G5" s="41" t="n">
         <v>46212</v>
       </c>
-      <c r="H5" s="20" t="s">
-        <v>149</v>
+      <c r="H5" s="27" t="s">
+        <v>163</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>150</v>
+        <v>164</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="36" t="n">
+      <c r="A6" s="41" t="n">
         <v>46223</v>
       </c>
       <c r="B6" s="8" t="s">
         <v>23</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>153</v>
-      </c>
-      <c r="F6" s="21" t="n">
+        <v>167</v>
+      </c>
+      <c r="F6" s="28" t="n">
         <v>311.98</v>
       </c>
-      <c r="G6" s="36" t="n">
+      <c r="G6" s="41" t="n">
         <v>46223</v>
       </c>
-      <c r="H6" s="20" t="s">
-        <v>154</v>
+      <c r="H6" s="27" t="s">
+        <v>168</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="36" t="n">
+      <c r="A7" s="41" t="n">
         <v>46223</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>19</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>156</v>
-      </c>
-      <c r="F7" s="21" t="n">
+        <v>170</v>
+      </c>
+      <c r="F7" s="28" t="n">
         <v>111.71</v>
       </c>
-      <c r="G7" s="36" t="n">
+      <c r="G7" s="41" t="n">
         <v>46223</v>
       </c>
-      <c r="H7" s="20" t="s">
-        <v>154</v>
+      <c r="H7" s="27" t="s">
+        <v>168</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="36" t="n">
+      <c r="A8" s="41" t="n">
         <v>46223</v>
       </c>
       <c r="B8" s="8" t="s">
         <v>19</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>158</v>
+        <v>46</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>160</v>
-      </c>
-      <c r="F8" s="21" t="n">
+        <v>173</v>
+      </c>
+      <c r="F8" s="28" t="n">
         <v>937.5</v>
       </c>
-      <c r="G8" s="36" t="n">
+      <c r="G8" s="41" t="n">
         <v>46223</v>
       </c>
-      <c r="H8" s="20" t="s">
-        <v>159</v>
+      <c r="H8" s="27" t="s">
+        <v>172</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="36" t="n">
+      <c r="A9" s="41" t="n">
         <v>46227</v>
       </c>
       <c r="B9" s="8" t="s">
@@ -2808,84 +3015,84 @@
         <v>14</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="F9" s="21" t="n">
+        <v>176</v>
+      </c>
+      <c r="F9" s="28" t="n">
         <v>3088.3</v>
       </c>
-      <c r="G9" s="36" t="n">
+      <c r="G9" s="41" t="n">
         <v>46227</v>
       </c>
-      <c r="H9" s="20" t="s">
-        <v>164</v>
+      <c r="H9" s="27" t="s">
+        <v>177</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="36" t="n">
+      <c r="A10" s="41" t="n">
         <v>46225</v>
       </c>
       <c r="B10" s="8" t="s">
         <v>23</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="E10" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="F10" s="28" t="n">
+        <v>162.96</v>
+      </c>
+      <c r="G10" s="41" t="n">
+        <v>46225</v>
+      </c>
+      <c r="H10" s="27" t="s">
         <v>168</v>
       </c>
-      <c r="F10" s="21" t="n">
-        <v>162.96</v>
-      </c>
-      <c r="G10" s="36" t="n">
-        <v>46225</v>
-      </c>
-      <c r="H10" s="20" t="s">
-        <v>154</v>
-      </c>
       <c r="I10" s="8" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="36" t="n">
+      <c r="A11" s="41" t="n">
         <v>46238</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>23</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>151</v>
+        <v>165</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="F11" s="21" t="n">
+        <v>184</v>
+      </c>
+      <c r="F11" s="28" t="n">
         <v>148.53</v>
       </c>
-      <c r="G11" s="36" t="n">
+      <c r="G11" s="41" t="n">
         <v>46238</v>
       </c>
-      <c r="H11" s="20" t="s">
-        <v>154</v>
+      <c r="H11" s="27" t="s">
+        <v>168</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="36" t="n">
+      <c r="A12" s="41" t="n">
         <v>46241</v>
       </c>
       <c r="B12" s="8" t="s">
@@ -2895,166 +3102,202 @@
         <v>14</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>173</v>
-      </c>
-      <c r="F12" s="21" t="n">
+        <v>186</v>
+      </c>
+      <c r="F12" s="28" t="n">
         <v>1710</v>
       </c>
-      <c r="G12" s="36" t="n">
+      <c r="G12" s="41" t="n">
         <v>46241</v>
       </c>
-      <c r="H12" s="20" t="s">
-        <v>159</v>
+      <c r="H12" s="27" t="s">
+        <v>172</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="37"/>
-      <c r="B13" s="38"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="38"/>
-      <c r="E13" s="38"/>
-      <c r="F13" s="39"/>
-      <c r="G13" s="37"/>
-      <c r="H13" s="38"/>
-      <c r="I13" s="38"/>
+      <c r="A13" s="41" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="F13" s="28" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="G13" s="41" t="n">
+        <v>46244</v>
+      </c>
+      <c r="H13" s="27" t="s">
+        <v>190</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="37"/>
-      <c r="B14" s="38"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="38"/>
-      <c r="F14" s="39"/>
-      <c r="G14" s="37"/>
-      <c r="H14" s="38"/>
-      <c r="I14" s="38"/>
+      <c r="A14" s="41" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="F14" s="28" t="n">
+        <v>344.16</v>
+      </c>
+      <c r="G14" s="41" t="n">
+        <v>46244</v>
+      </c>
+      <c r="H14" s="27" t="s">
+        <v>190</v>
+      </c>
+      <c r="I14" s="8" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="37"/>
-      <c r="B15" s="38"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="38"/>
-      <c r="E15" s="38"/>
-      <c r="F15" s="39"/>
-      <c r="G15" s="37"/>
-      <c r="H15" s="38"/>
-      <c r="I15" s="38"/>
+      <c r="A15" s="42"/>
+      <c r="B15" s="43"/>
+      <c r="C15" s="43"/>
+      <c r="D15" s="43"/>
+      <c r="E15" s="43"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="43"/>
+      <c r="I15" s="43"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="37"/>
-      <c r="B16" s="38"/>
-      <c r="C16" s="38"/>
-      <c r="D16" s="38"/>
-      <c r="E16" s="38"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="37"/>
-      <c r="H16" s="38"/>
-      <c r="I16" s="38"/>
+      <c r="A16" s="42"/>
+      <c r="B16" s="43"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="43"/>
+      <c r="F16" s="44"/>
+      <c r="G16" s="42"/>
+      <c r="H16" s="43"/>
+      <c r="I16" s="43"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="37"/>
-      <c r="B17" s="38"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="38"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="37"/>
-      <c r="H17" s="38"/>
-      <c r="I17" s="38"/>
+      <c r="A17" s="42"/>
+      <c r="B17" s="43"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="43"/>
+      <c r="F17" s="44"/>
+      <c r="G17" s="42"/>
+      <c r="H17" s="43"/>
+      <c r="I17" s="43"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="37"/>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="38"/>
-      <c r="I18" s="38"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="43"/>
+      <c r="E18" s="43"/>
+      <c r="F18" s="44"/>
+      <c r="G18" s="42"/>
+      <c r="H18" s="43"/>
+      <c r="I18" s="43"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="37"/>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="37"/>
-      <c r="H19" s="38"/>
-      <c r="I19" s="38"/>
+      <c r="A19" s="42"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="43"/>
+      <c r="E19" s="43"/>
+      <c r="F19" s="44"/>
+      <c r="G19" s="42"/>
+      <c r="H19" s="43"/>
+      <c r="I19" s="43"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="37"/>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="39"/>
-      <c r="G20" s="37"/>
-      <c r="H20" s="38"/>
-      <c r="I20" s="38"/>
+      <c r="A20" s="42"/>
+      <c r="B20" s="43"/>
+      <c r="C20" s="43"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="43"/>
+      <c r="F20" s="44"/>
+      <c r="G20" s="42"/>
+      <c r="H20" s="43"/>
+      <c r="I20" s="43"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="37"/>
-      <c r="B21" s="38"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="39"/>
-      <c r="G21" s="37"/>
-      <c r="H21" s="38"/>
-      <c r="I21" s="38"/>
+      <c r="A21" s="42"/>
+      <c r="B21" s="43"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="43"/>
+      <c r="F21" s="44"/>
+      <c r="G21" s="42"/>
+      <c r="H21" s="43"/>
+      <c r="I21" s="43"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="37"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="39"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="38"/>
-      <c r="I22" s="38"/>
+      <c r="A22" s="42"/>
+      <c r="B22" s="43"/>
+      <c r="C22" s="43"/>
+      <c r="D22" s="43"/>
+      <c r="E22" s="43"/>
+      <c r="F22" s="44"/>
+      <c r="G22" s="42"/>
+      <c r="H22" s="43"/>
+      <c r="I22" s="43"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="37"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="39"/>
-      <c r="G23" s="37"/>
-      <c r="H23" s="38"/>
-      <c r="I23" s="38"/>
+      <c r="A23" s="42"/>
+      <c r="B23" s="43"/>
+      <c r="C23" s="43"/>
+      <c r="D23" s="43"/>
+      <c r="E23" s="43"/>
+      <c r="F23" s="44"/>
+      <c r="G23" s="42"/>
+      <c r="H23" s="43"/>
+      <c r="I23" s="43"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="37"/>
-      <c r="B24" s="38"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="39"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="38"/>
-      <c r="I24" s="38"/>
+      <c r="A24" s="42"/>
+      <c r="B24" s="43"/>
+      <c r="C24" s="43"/>
+      <c r="D24" s="43"/>
+      <c r="E24" s="43"/>
+      <c r="F24" s="44"/>
+      <c r="G24" s="42"/>
+      <c r="H24" s="43"/>
+      <c r="I24" s="43"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="37"/>
-      <c r="B25" s="38"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="39"/>
-      <c r="G25" s="37"/>
-      <c r="H25" s="38"/>
-      <c r="I25" s="38"/>
+      <c r="A25" s="42"/>
+      <c r="B25" s="43"/>
+      <c r="C25" s="43"/>
+      <c r="D25" s="43"/>
+      <c r="E25" s="43"/>
+      <c r="F25" s="44"/>
+      <c r="G25" s="42"/>
+      <c r="H25" s="43"/>
+      <c r="I25" s="43"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3077,280 +3320,260 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>175</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>176</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="B4" s="40" t="n">
-        <v>1130</v>
+        <v>198</v>
+      </c>
+      <c r="B4" s="45" t="n">
+        <v>1360</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="D4" s="41" t="n">
+        <v>199</v>
+      </c>
+      <c r="D4" s="46" t="n">
         <f aca="false">B4-SUM(E8:E40)</f>
-        <v>506.53</v>
+        <v>1015.84</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>179</v>
+        <v>200</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>180</v>
+        <v>201</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>181</v>
+        <v>202</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>182</v>
+        <v>203</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>183</v>
+        <v>204</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="36" t="n">
-        <v>46223</v>
+        <v>205</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="41" t="n">
+        <v>46244</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>151</v>
+        <v>192</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="D8" s="20" t="s">
-        <v>186</v>
-      </c>
-      <c r="E8" s="21" t="n">
-        <v>311.98</v>
+        <v>206</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="E8" s="28" t="n">
+        <v>344.16</v>
       </c>
       <c r="F8" s="10" t="n">
         <f aca="false">IF(E8="","",$B$4-SUM($E$8:E8))</f>
-        <v>818.02</v>
+        <v>1015.84</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="36" t="n">
-        <v>46225</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>187</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>188</v>
-      </c>
-      <c r="E9" s="21" t="n">
-        <v>162.96</v>
-      </c>
-      <c r="F9" s="10" t="n">
+      <c r="A9" s="42"/>
+      <c r="B9" s="43"/>
+      <c r="C9" s="43"/>
+      <c r="D9" s="43"/>
+      <c r="E9" s="44"/>
+      <c r="F9" s="10" t="str">
         <f aca="false">IF(E9="","",$B$4-SUM($E$8:E9))</f>
-        <v>655.06</v>
+        <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="36" t="n">
-        <v>46238</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>189</v>
-      </c>
-      <c r="D10" s="20" t="s">
-        <v>190</v>
-      </c>
-      <c r="E10" s="21" t="n">
-        <v>148.53</v>
-      </c>
-      <c r="F10" s="10" t="n">
+      <c r="A10" s="42"/>
+      <c r="B10" s="43"/>
+      <c r="C10" s="43"/>
+      <c r="D10" s="43"/>
+      <c r="E10" s="44"/>
+      <c r="F10" s="10" t="str">
         <f aca="false">IF(E10="","",$B$4-SUM($E$8:E10))</f>
-        <v>506.53</v>
+        <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="37"/>
-      <c r="B11" s="38"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="38"/>
-      <c r="E11" s="39"/>
+      <c r="A11" s="42"/>
+      <c r="B11" s="43"/>
+      <c r="C11" s="43"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="44"/>
       <c r="F11" s="10" t="str">
         <f aca="false">IF(E11="","",$B$4-SUM($E$8:E11))</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="37"/>
-      <c r="B12" s="38"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="38"/>
-      <c r="E12" s="39"/>
+      <c r="A12" s="42"/>
+      <c r="B12" s="43"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="44"/>
       <c r="F12" s="10" t="str">
         <f aca="false">IF(E12="","",$B$4-SUM($E$8:E12))</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="37"/>
-      <c r="B13" s="38"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="38"/>
-      <c r="E13" s="39"/>
+      <c r="A13" s="42"/>
+      <c r="B13" s="43"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="43"/>
+      <c r="E13" s="44"/>
       <c r="F13" s="10" t="str">
         <f aca="false">IF(E13="","",$B$4-SUM($E$8:E13))</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="37"/>
-      <c r="B14" s="38"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="38"/>
-      <c r="E14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="43"/>
+      <c r="C14" s="43"/>
+      <c r="D14" s="43"/>
+      <c r="E14" s="44"/>
       <c r="F14" s="10" t="str">
         <f aca="false">IF(E14="","",$B$4-SUM($E$8:E14))</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="37"/>
-      <c r="B15" s="38"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="38"/>
-      <c r="E15" s="39"/>
+      <c r="A15" s="42"/>
+      <c r="B15" s="43"/>
+      <c r="C15" s="43"/>
+      <c r="D15" s="43"/>
+      <c r="E15" s="44"/>
       <c r="F15" s="10" t="str">
         <f aca="false">IF(E15="","",$B$4-SUM($E$8:E15))</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="37"/>
-      <c r="B16" s="38"/>
-      <c r="C16" s="38"/>
-      <c r="D16" s="38"/>
-      <c r="E16" s="39"/>
+      <c r="A16" s="42"/>
+      <c r="B16" s="43"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="44"/>
       <c r="F16" s="10" t="str">
         <f aca="false">IF(E16="","",$B$4-SUM($E$8:E16))</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="37"/>
-      <c r="B17" s="38"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="39"/>
+      <c r="A17" s="42"/>
+      <c r="B17" s="43"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="44"/>
       <c r="F17" s="10" t="str">
         <f aca="false">IF(E17="","",$B$4-SUM($E$8:E17))</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="37"/>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="43"/>
+      <c r="E18" s="44"/>
       <c r="F18" s="10" t="str">
         <f aca="false">IF(E18="","",$B$4-SUM($E$8:E18))</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="37"/>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="39"/>
+      <c r="A19" s="42"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="43"/>
+      <c r="E19" s="44"/>
       <c r="F19" s="10" t="str">
         <f aca="false">IF(E19="","",$B$4-SUM($E$8:E19))</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="37"/>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="39"/>
+      <c r="A20" s="42"/>
+      <c r="B20" s="43"/>
+      <c r="C20" s="43"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="44"/>
       <c r="F20" s="10" t="str">
         <f aca="false">IF(E20="","",$B$4-SUM($E$8:E20))</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="37"/>
-      <c r="B21" s="38"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="39"/>
+      <c r="A21" s="42"/>
+      <c r="B21" s="43"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="44"/>
       <c r="F21" s="10" t="str">
         <f aca="false">IF(E21="","",$B$4-SUM($E$8:E21))</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="37"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="39"/>
+      <c r="A22" s="42"/>
+      <c r="B22" s="43"/>
+      <c r="C22" s="43"/>
+      <c r="D22" s="43"/>
+      <c r="E22" s="44"/>
       <c r="F22" s="10" t="str">
         <f aca="false">IF(E22="","",$B$4-SUM($E$8:E22))</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="37"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="39"/>
+      <c r="A23" s="42"/>
+      <c r="B23" s="43"/>
+      <c r="C23" s="43"/>
+      <c r="D23" s="43"/>
+      <c r="E23" s="44"/>
       <c r="F23" s="10" t="str">
         <f aca="false">IF(E23="","",$B$4-SUM($E$8:E23))</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="37"/>
-      <c r="B24" s="38"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="39"/>
+      <c r="A24" s="42"/>
+      <c r="B24" s="43"/>
+      <c r="C24" s="43"/>
+      <c r="D24" s="43"/>
+      <c r="E24" s="44"/>
       <c r="F24" s="10" t="str">
         <f aca="false">IF(E24="","",$B$4-SUM($E$8:E24))</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="37"/>
-      <c r="B25" s="38"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="39"/>
+      <c r="A25" s="42"/>
+      <c r="B25" s="43"/>
+      <c r="C25" s="43"/>
+      <c r="D25" s="43"/>
+      <c r="E25" s="44"/>
       <c r="F25" s="10" t="str">
         <f aca="false">IF(E25="","",$B$4-SUM($E$8:E25))</f>
         <v/>
@@ -3372,6 +3595,306 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="5" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="B4" s="45" t="n">
+        <v>1130</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="D4" s="46" t="n">
+        <f aca="false">B4-SUM(E8:E40)</f>
+        <v>506.53</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="41" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="D8" s="27" t="s">
+        <v>213</v>
+      </c>
+      <c r="E8" s="28" t="n">
+        <v>311.98</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <f aca="false">IF(E8="","",$B$4-SUM($E$8:E8))</f>
+        <v>818.02</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="41" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D9" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="E9" s="28" t="n">
+        <v>162.96</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <f aca="false">IF(E9="","",$B$4-SUM($E$8:E9))</f>
+        <v>655.06</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="41" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="D10" s="27" t="s">
+        <v>217</v>
+      </c>
+      <c r="E10" s="28" t="n">
+        <v>148.53</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <f aca="false">IF(E10="","",$B$4-SUM($E$8:E10))</f>
+        <v>506.53</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="42"/>
+      <c r="B11" s="43"/>
+      <c r="C11" s="43"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="44"/>
+      <c r="F11" s="10" t="str">
+        <f aca="false">IF(E11="","",$B$4-SUM($E$8:E11))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="42"/>
+      <c r="B12" s="43"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43"/>
+      <c r="E12" s="44"/>
+      <c r="F12" s="10" t="str">
+        <f aca="false">IF(E12="","",$B$4-SUM($E$8:E12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="42"/>
+      <c r="B13" s="43"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="43"/>
+      <c r="E13" s="44"/>
+      <c r="F13" s="10" t="str">
+        <f aca="false">IF(E13="","",$B$4-SUM($E$8:E13))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="42"/>
+      <c r="B14" s="43"/>
+      <c r="C14" s="43"/>
+      <c r="D14" s="43"/>
+      <c r="E14" s="44"/>
+      <c r="F14" s="10" t="str">
+        <f aca="false">IF(E14="","",$B$4-SUM($E$8:E14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="42"/>
+      <c r="B15" s="43"/>
+      <c r="C15" s="43"/>
+      <c r="D15" s="43"/>
+      <c r="E15" s="44"/>
+      <c r="F15" s="10" t="str">
+        <f aca="false">IF(E15="","",$B$4-SUM($E$8:E15))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="42"/>
+      <c r="B16" s="43"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="44"/>
+      <c r="F16" s="10" t="str">
+        <f aca="false">IF(E16="","",$B$4-SUM($E$8:E16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="42"/>
+      <c r="B17" s="43"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="43"/>
+      <c r="E17" s="44"/>
+      <c r="F17" s="10" t="str">
+        <f aca="false">IF(E17="","",$B$4-SUM($E$8:E17))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="42"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="43"/>
+      <c r="E18" s="44"/>
+      <c r="F18" s="10" t="str">
+        <f aca="false">IF(E18="","",$B$4-SUM($E$8:E18))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="42"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="43"/>
+      <c r="E19" s="44"/>
+      <c r="F19" s="10" t="str">
+        <f aca="false">IF(E19="","",$B$4-SUM($E$8:E19))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="42"/>
+      <c r="B20" s="43"/>
+      <c r="C20" s="43"/>
+      <c r="D20" s="43"/>
+      <c r="E20" s="44"/>
+      <c r="F20" s="10" t="str">
+        <f aca="false">IF(E20="","",$B$4-SUM($E$8:E20))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="42"/>
+      <c r="B21" s="43"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="44"/>
+      <c r="F21" s="10" t="str">
+        <f aca="false">IF(E21="","",$B$4-SUM($E$8:E21))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="42"/>
+      <c r="B22" s="43"/>
+      <c r="C22" s="43"/>
+      <c r="D22" s="43"/>
+      <c r="E22" s="44"/>
+      <c r="F22" s="10" t="str">
+        <f aca="false">IF(E22="","",$B$4-SUM($E$8:E22))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="42"/>
+      <c r="B23" s="43"/>
+      <c r="C23" s="43"/>
+      <c r="D23" s="43"/>
+      <c r="E23" s="44"/>
+      <c r="F23" s="10" t="str">
+        <f aca="false">IF(E23="","",$B$4-SUM($E$8:E23))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="42"/>
+      <c r="B24" s="43"/>
+      <c r="C24" s="43"/>
+      <c r="D24" s="43"/>
+      <c r="E24" s="44"/>
+      <c r="F24" s="10" t="str">
+        <f aca="false">IF(E24="","",$B$4-SUM($E$8:E24))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="42"/>
+      <c r="B25" s="43"/>
+      <c r="C25" s="43"/>
+      <c r="D25" s="43"/>
+      <c r="E25" s="44"/>
+      <c r="F25" s="10" t="str">
+        <f aca="false">IF(E25="","",$B$4-SUM($E$8:E25))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:E25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -3383,221 +3906,221 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>191</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>192</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="B4" s="40" t="n">
+        <v>220</v>
+      </c>
+      <c r="B4" s="45" t="n">
         <v>5000</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="D4" s="41" t="n">
+        <v>199</v>
+      </c>
+      <c r="D4" s="46" t="n">
         <f aca="false">B4-SUM(D8:D40)</f>
         <v>5000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>179</v>
+        <v>200</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>194</v>
+        <v>221</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>195</v>
+        <v>222</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>183</v>
+        <v>204</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>184</v>
+        <v>205</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="37"/>
-      <c r="B8" s="38"/>
-      <c r="C8" s="38"/>
-      <c r="D8" s="39"/>
+      <c r="A8" s="42"/>
+      <c r="B8" s="43"/>
+      <c r="C8" s="43"/>
+      <c r="D8" s="44"/>
       <c r="E8" s="10" t="str">
         <f aca="false">IF(D8="","",$B$4-SUM($D$8:D8))</f>
         <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="37"/>
-      <c r="B9" s="38"/>
-      <c r="C9" s="38"/>
-      <c r="D9" s="39"/>
+      <c r="A9" s="42"/>
+      <c r="B9" s="43"/>
+      <c r="C9" s="43"/>
+      <c r="D9" s="44"/>
       <c r="E9" s="10" t="str">
         <f aca="false">IF(D9="","",$B$4-SUM($D$8:D9))</f>
         <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="37"/>
-      <c r="B10" s="38"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="39"/>
+      <c r="A10" s="42"/>
+      <c r="B10" s="43"/>
+      <c r="C10" s="43"/>
+      <c r="D10" s="44"/>
       <c r="E10" s="10" t="str">
         <f aca="false">IF(D10="","",$B$4-SUM($D$8:D10))</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="37"/>
-      <c r="B11" s="38"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="39"/>
+      <c r="A11" s="42"/>
+      <c r="B11" s="43"/>
+      <c r="C11" s="43"/>
+      <c r="D11" s="44"/>
       <c r="E11" s="10" t="str">
         <f aca="false">IF(D11="","",$B$4-SUM($D$8:D11))</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="37"/>
-      <c r="B12" s="38"/>
-      <c r="C12" s="38"/>
-      <c r="D12" s="39"/>
+      <c r="A12" s="42"/>
+      <c r="B12" s="43"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="44"/>
       <c r="E12" s="10" t="str">
         <f aca="false">IF(D12="","",$B$4-SUM($D$8:D12))</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="37"/>
-      <c r="B13" s="38"/>
-      <c r="C13" s="38"/>
-      <c r="D13" s="39"/>
+      <c r="A13" s="42"/>
+      <c r="B13" s="43"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="44"/>
       <c r="E13" s="10" t="str">
         <f aca="false">IF(D13="","",$B$4-SUM($D$8:D13))</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="37"/>
-      <c r="B14" s="38"/>
-      <c r="C14" s="38"/>
-      <c r="D14" s="39"/>
+      <c r="A14" s="42"/>
+      <c r="B14" s="43"/>
+      <c r="C14" s="43"/>
+      <c r="D14" s="44"/>
       <c r="E14" s="10" t="str">
         <f aca="false">IF(D14="","",$B$4-SUM($D$8:D14))</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="37"/>
-      <c r="B15" s="38"/>
-      <c r="C15" s="38"/>
-      <c r="D15" s="39"/>
+      <c r="A15" s="42"/>
+      <c r="B15" s="43"/>
+      <c r="C15" s="43"/>
+      <c r="D15" s="44"/>
       <c r="E15" s="10" t="str">
         <f aca="false">IF(D15="","",$B$4-SUM($D$8:D15))</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="37"/>
-      <c r="B16" s="38"/>
-      <c r="C16" s="38"/>
-      <c r="D16" s="39"/>
+      <c r="A16" s="42"/>
+      <c r="B16" s="43"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="44"/>
       <c r="E16" s="10" t="str">
         <f aca="false">IF(D16="","",$B$4-SUM($D$8:D16))</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="37"/>
-      <c r="B17" s="38"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="39"/>
+      <c r="A17" s="42"/>
+      <c r="B17" s="43"/>
+      <c r="C17" s="43"/>
+      <c r="D17" s="44"/>
       <c r="E17" s="10" t="str">
         <f aca="false">IF(D17="","",$B$4-SUM($D$8:D17))</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="37"/>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="39"/>
+      <c r="A18" s="42"/>
+      <c r="B18" s="43"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="44"/>
       <c r="E18" s="10" t="str">
         <f aca="false">IF(D18="","",$B$4-SUM($D$8:D18))</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="37"/>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="39"/>
+      <c r="A19" s="42"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="44"/>
       <c r="E19" s="10" t="str">
         <f aca="false">IF(D19="","",$B$4-SUM($D$8:D19))</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="37"/>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="39"/>
+      <c r="A20" s="42"/>
+      <c r="B20" s="43"/>
+      <c r="C20" s="43"/>
+      <c r="D20" s="44"/>
       <c r="E20" s="10" t="str">
         <f aca="false">IF(D20="","",$B$4-SUM($D$8:D20))</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="37"/>
-      <c r="B21" s="38"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="39"/>
+      <c r="A21" s="42"/>
+      <c r="B21" s="43"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="44"/>
       <c r="E21" s="10" t="str">
         <f aca="false">IF(D21="","",$B$4-SUM($D$8:D21))</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="37"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="39"/>
+      <c r="A22" s="42"/>
+      <c r="B22" s="43"/>
+      <c r="C22" s="43"/>
+      <c r="D22" s="44"/>
       <c r="E22" s="10" t="str">
         <f aca="false">IF(D22="","",$B$4-SUM($D$8:D22))</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="37"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="39"/>
+      <c r="A23" s="42"/>
+      <c r="B23" s="43"/>
+      <c r="C23" s="43"/>
+      <c r="D23" s="44"/>
       <c r="E23" s="10" t="str">
         <f aca="false">IF(D23="","",$B$4-SUM($D$8:D23))</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="37"/>
-      <c r="B24" s="38"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="39"/>
+      <c r="A24" s="42"/>
+      <c r="B24" s="43"/>
+      <c r="C24" s="43"/>
+      <c r="D24" s="44"/>
       <c r="E24" s="10" t="str">
         <f aca="false">IF(D24="","",$B$4-SUM($D$8:D24))</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="37"/>
-      <c r="B25" s="38"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="39"/>
+      <c r="A25" s="42"/>
+      <c r="B25" s="43"/>
+      <c r="C25" s="43"/>
+      <c r="D25" s="44"/>
       <c r="E25" s="10" t="str">
         <f aca="false">IF(D25="","",$B$4-SUM($D$8:D25))</f>
         <v/>

</xml_diff>